<commit_message>
feat: students and classes worksheets combined
</commit_message>
<xml_diff>
--- a/web/app/spreadsheet_templates/students_export_template.xlsx
+++ b/web/app/spreadsheet_templates/students_export_template.xlsx
@@ -7,10 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tentang Ekspor" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="students" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="classes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'instructions'!$A$1:$H$48</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
@@ -142,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -358,6 +361,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFEFCFD2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFEFCFD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFEFCFD2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFEFCFD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -369,7 +401,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -508,6 +540,41 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -664,15 +731,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StudentsExportTable" displayName="StudentsExportTable" ref="A1:F2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F2"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StudentsExportTable" displayName="StudentsExportTable" ref="A1:H2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:H2"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="NAMA"/>
-    <tableColumn id="3" name="ID KELAS"/>
-    <tableColumn id="4" name="NISN"/>
-    <tableColumn id="5" name="STATUS"/>
-    <tableColumn id="6" name="NOMOR WALI"/>
+    <tableColumn id="3" name="NISN"/>
+    <tableColumn id="4" name="STATUS"/>
+    <tableColumn id="5" name="NOMOR WALI"/>
+    <tableColumn id="6" name="JENJANG"/>
+    <tableColumn id="7" name="NAMA KELAS"/>
+    <tableColumn id="8" name="ID KELAS"/>
+  </tableColumns>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClassesExportTable" displayName="ClassesExportTable" ref="A1:C2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:C2"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="ID KELAS"/>
+    <tableColumn id="2" name="JENJANG"/>
+    <tableColumn id="3" name="NAMA KELAS"/>
   </tableColumns>
 </table>
 </file>
@@ -853,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.7578125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3.42" customWidth="1" style="21" min="1" max="1"/>
@@ -876,7 +956,7 @@
       <c r="A2" s="23" t="n"/>
       <c r="B2" s="24" t="inlineStr">
         <is>
-          <t>Ekspor &amp; Impor Data Siswa</t>
+          <t>Ekspor &amp; Impor Siswa dan Kelas</t>
         </is>
       </c>
       <c r="G2" s="25" t="inlineStr">
@@ -914,7 +994,7 @@
       <c r="A5" s="23" t="n"/>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Template ekspor dan impor untuk mengedit data lama atau membuat data baru.</t>
+          <t>Workbook ini dibuat oleh Absensa untuk ekspor serta penyuntingan massal dan impor kembali.</t>
         </is>
       </c>
     </row>
@@ -982,7 +1062,7 @@
       <c r="C9" s="26" t="n"/>
       <c r="D9" s="32" t="inlineStr">
         <is>
-          <t>students</t>
+          <t>students dan classes</t>
         </is>
       </c>
       <c r="E9" s="28" t="n"/>
@@ -1000,7 +1080,7 @@
       <c r="C10" s="26" t="n"/>
       <c r="D10" s="33" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>ID siswa dan ID KELAS (dilindungi)</t>
         </is>
       </c>
       <c r="E10" s="28" t="n"/>
@@ -1018,11 +1098,11 @@
       <c r="G11" s="23" t="n"/>
       <c r="H11" s="23" t="n"/>
     </row>
-    <row r="12" ht="23" customHeight="1" s="22">
+    <row r="12" ht="24" customHeight="1" s="22">
       <c r="A12" s="23" t="n"/>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>Mengedit atau menambah data</t>
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>Isi workbook</t>
         </is>
       </c>
       <c r="C12" s="28" t="n"/>
@@ -1032,21 +1112,17 @@
       <c r="G12" s="28" t="n"/>
       <c r="H12" s="26" t="n"/>
     </row>
-    <row r="13" ht="34" customHeight="1" s="22">
+    <row r="13" ht="62" customHeight="1" s="22">
       <c r="A13" s="23" t="n"/>
       <c r="B13" s="29" t="inlineStr">
         <is>
-          <t>1. Edit data yang sudah ada: ubah kolom yang diperlukan dan pertahankan ID aslinya.</t>
+          <t>students berisi data siswa sesuai filter ekspor di atas. classes selalu berisi seluruh kelas dari semua jenjang, tanpa mengikuti filter siswa, dan menjadi sumber pilihan dropdown.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1" s="22">
       <c r="A14" s="23" t="n"/>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>2. Buat siswa baru: isi baris kosong di bawah data terakhir dan biarkan ID kosong.</t>
-        </is>
-      </c>
+      <c r="B14" s="29" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="23" t="n"/>
@@ -1058,11 +1134,11 @@
       <c r="G15" s="23" t="n"/>
       <c r="H15" s="23" t="n"/>
     </row>
-    <row r="16" ht="23" customHeight="1" s="22">
+    <row r="16" ht="24" customHeight="1" s="22">
       <c r="A16" s="23" t="n"/>
-      <c r="B16" s="27" t="inlineStr">
-        <is>
-          <t>Sebelum mengimpor</t>
+      <c r="B16" s="53" t="inlineStr">
+        <is>
+          <t>Jangan mengubah identitas</t>
         </is>
       </c>
       <c r="C16" s="28" t="n"/>
@@ -1072,33 +1148,23 @@
       <c r="G16" s="28" t="n"/>
       <c r="H16" s="26" t="n"/>
     </row>
-    <row r="17" ht="34" customHeight="1" s="22">
+    <row r="17" ht="62" customHeight="1" s="22">
       <c r="A17" s="23" t="n"/>
-      <c r="B17" s="34" t="inlineStr">
-        <is>
-          <t>1. Jangan mengubah nama sheet atau judul kolom. Baris kosong bukan data baru.</t>
-        </is>
-      </c>
-      <c r="C17" s="35" t="n"/>
-      <c r="D17" s="35" t="n"/>
-      <c r="E17" s="35" t="n"/>
-      <c r="F17" s="35" t="n"/>
-      <c r="G17" s="35" t="n"/>
-      <c r="H17" s="36" t="n"/>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>Jangan mengganti nama sheet atau judul kolom. ID siswa mengidentifikasi siswa; ID KELAS mengidentifikasi kelas. ID dilindungi dan tidak boleh diubah. Di students, ID kelas disembunyikan sebagai metadata internal; Anda tidak perlu mengetahui atau mengeditnya.</t>
+        </is>
+      </c>
+      <c r="C17" s="63" t="n"/>
+      <c r="D17" s="63" t="n"/>
+      <c r="E17" s="63" t="n"/>
+      <c r="F17" s="63" t="n"/>
+      <c r="G17" s="63" t="n"/>
+      <c r="H17" s="64" t="n"/>
     </row>
     <row r="18" ht="34" customHeight="1" s="22">
       <c r="A18" s="23" t="n"/>
-      <c r="B18" s="34" t="inlineStr">
-        <is>
-          <t>2. Simpan sebagai .xlsx. ID terisi untuk pembaruan; ID kosong untuk pembuatan data.</t>
-        </is>
-      </c>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="35" t="n"/>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="36" t="n"/>
+      <c r="B18" s="34" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="22">
       <c r="A19" s="23" t="n"/>
@@ -1110,11 +1176,11 @@
       <c r="G19" s="23" t="n"/>
       <c r="H19" s="23" t="n"/>
     </row>
-    <row r="20" ht="23" customHeight="1" s="22">
+    <row r="20" ht="24" customHeight="1" s="22">
       <c r="A20" s="23" t="n"/>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>Mengisi baris baru</t>
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>Menentukan kelas siswa</t>
         </is>
       </c>
       <c r="C20" s="28" t="n"/>
@@ -1124,29 +1190,22 @@
       <c r="G20" s="28" t="n"/>
       <c r="H20" s="26" t="n"/>
     </row>
-    <row r="21" ht="64" customHeight="1" s="22">
+    <row r="21" ht="62" customHeight="1" s="22">
       <c r="A21" s="23" t="n"/>
-      <c r="B21" s="37" t="inlineStr">
-        <is>
-          <t>Validasi tersedia sampai baris terakhir sheet. NISN: tepat 10 digit (termasuk nol di depan). STATUS: pilih Aktif atau Tidak aktif. ID KELAS boleh kosong jika belum memiliki kelas. NOMOR WALI opsional: angka saja, diawali 08 atau 628, maksimal 32 digit. Isi langsung pada baris kosong; saat menyalin data, tempel nilai saja agar format dan validasi tetap terjaga.</t>
-        </is>
-      </c>
-      <c r="C21" s="38" t="n"/>
-      <c r="D21" s="38" t="n"/>
-      <c r="E21" s="38" t="n"/>
-      <c r="F21" s="38" t="n"/>
-      <c r="G21" s="38" t="n"/>
-      <c r="H21" s="39" t="n"/>
+      <c r="B21" s="65" t="inlineStr">
+        <is>
+          <t>Di students, pilih JENJANG dan NAMA KELAS melalui dropdown. Pilihan berasal dari classes. Untuk siswa baru, keduanya wajib diisi dan kelas harus tercantum pada classes. Untuk siswa lama, kosongkan kedua nilai jika ingin melepas kelas. Nilai yang hanya terisi sebagian ditolak.</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="42" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1" s="22">
       <c r="A22" s="23" t="n"/>
-      <c r="B22" s="40" t="n"/>
-      <c r="C22" s="41" t="n"/>
-      <c r="D22" s="41" t="n"/>
-      <c r="E22" s="41" t="n"/>
-      <c r="F22" s="41" t="n"/>
-      <c r="G22" s="41" t="n"/>
-      <c r="H22" s="42" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="22">
       <c r="A23" s="23" t="n"/>
@@ -1158,40 +1217,161 @@
       <c r="G23" s="23" t="n"/>
       <c r="H23" s="23" t="n"/>
     </row>
-    <row r="24" ht="15" customHeight="1" s="22">
+    <row r="24" ht="24" customHeight="1" s="22">
       <c r="A24" s="23" t="n"/>
-      <c r="B24" s="43" t="n"/>
-      <c r="C24" s="43" t="n"/>
-      <c r="D24" s="43" t="n"/>
-      <c r="E24" s="43" t="n"/>
-      <c r="F24" s="43" t="n"/>
-      <c r="G24" s="43" t="n"/>
-      <c r="H24" s="43" t="n"/>
+      <c r="B24" s="53" t="inlineStr">
+        <is>
+          <t>Membuat kelas hanya melalui classes</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="n"/>
+      <c r="D24" s="28" t="n"/>
+      <c r="E24" s="28" t="n"/>
+      <c r="F24" s="28" t="n"/>
+      <c r="G24" s="28" t="n"/>
+      <c r="H24" s="26" t="n"/>
+    </row>
+    <row r="25" ht="74" customHeight="1" s="22">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Tambahkan baris pada classes dengan ID KELAS kosong, lalu isi JENJANG dan NAMA KELAS. Siswa dapat merujuk pasangan itu dalam impor yang sama. Satu kelas baru akan dipakai bersama oleh semua siswa yang merujuknya. Salah ketik pada students tidak akan membuat kelas baru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1" s="22">
+      <c r="B28" s="53" t="inlineStr">
+        <is>
+          <t>Mengganti nama atau jenjang kelas</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="n"/>
+      <c r="D28" s="28" t="n"/>
+      <c r="E28" s="28" t="n"/>
+      <c r="F28" s="28" t="n"/>
+      <c r="G28" s="28" t="n"/>
+      <c r="H28" s="26" t="n"/>
+    </row>
+    <row r="29" ht="86" customHeight="1" s="22">
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>Edit JENJANG dan/atau NAMA KELAS pada classes dengan mempertahankan ID yang dilindungi. Contoh: 10 / IPA 1 menjadi 10 / IPA A. Siswa tetap mengikuti kelas yang sama meskipun nilai lama di students belum diedit; tidak perlu mengubah setiap siswa. Untuk memindahkan siswa, ubah pasangan jenjang dan nama kelasnya ke kelas lain yang tercantum pada classes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" s="22">
+      <c r="B32" s="53" t="inlineStr">
+        <is>
+          <t>Menghapus baris BUKAN menghapus kelas</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="n"/>
+      <c r="D32" s="28" t="n"/>
+      <c r="E32" s="28" t="n"/>
+      <c r="F32" s="28" t="n"/>
+      <c r="G32" s="28" t="n"/>
+      <c r="H32" s="26" t="n"/>
+    </row>
+    <row r="33" ht="62" customHeight="1" s="22">
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>Menghapus baris kelas hanya menghapusnya dari workbook dan pilihan kelasnya, bukan dari Absensa. Siswa yang masih merujuk kelas tersebut perlu disesuaikan atau baris kelas dikembalikan. Penghapusan kelas dari database dilakukan secara eksplisit melalui halaman/dashboard Kelas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" s="22">
+      <c r="B36" s="53" t="inlineStr">
+        <is>
+          <t>Impor bersifat semua-atau-tidak-sama-sekali</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="n"/>
+      <c r="D36" s="28" t="n"/>
+      <c r="E36" s="28" t="n"/>
+      <c r="F36" s="28" t="n"/>
+      <c r="G36" s="28" t="n"/>
+      <c r="H36" s="26" t="n"/>
+    </row>
+    <row r="37" ht="62" customHeight="1" s="22">
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>Absensa memvalidasi seluruh workbook sebelum menyimpan apa pun. Jika satu baris saja salah, seluruh impor ditolak: tidak ada siswa yang diubah dan tidak ada kelas yang diubah atau dibuat. Perbaiki semua kesalahan yang dilaporkan, lalu impor kembali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1" s="22">
+      <c r="B40" s="53" t="inlineStr">
+        <is>
+          <t>Mengisi data siswa</t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="n"/>
+      <c r="D40" s="28" t="n"/>
+      <c r="E40" s="28" t="n"/>
+      <c r="F40" s="28" t="n"/>
+      <c r="G40" s="28" t="n"/>
+      <c r="H40" s="26" t="n"/>
+    </row>
+    <row r="41" ht="62" customHeight="1" s="22">
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>Pertahankan ID siswa untuk pembaruan; kosongkan ID untuk siswa baru. NISN wajib tepat 10 digit dan disimpan sebagai teks agar nol di depan tidak hilang. STATUS: Aktif atau Tidak aktif. NOMOR WALI opsional, angka saja diawali 08 atau 628, maksimal 32 digit. Baris kosong diabaikan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1" s="22">
+      <c r="B44" s="53" t="inlineStr">
+        <is>
+          <t>Pilihan Excel dan baris baru</t>
+        </is>
+      </c>
+      <c r="C44" s="28" t="n"/>
+      <c r="D44" s="28" t="n"/>
+      <c r="E44" s="28" t="n"/>
+      <c r="F44" s="28" t="n"/>
+      <c r="G44" s="28" t="n"/>
+      <c r="H44" s="26" t="n"/>
+    </row>
+    <row r="45" ht="86" customHeight="1" s="22">
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>Dropdown memakai jenjang dan nama kelas dari classes saat file dibuat. Jika kelas baru belum muncul di pilihan, ketik nilainya setelah menambahkannya pada classes. Kombinasi jenjang dan nama kelas harus unik; jenjang 1–20 dan nama maksimal 20 karakter. Kolom data dapat diedit; ID dan metadata dilindungi. Tersedia 100 baris entri kosong. Simpan sebagai .xlsx tanpa makro.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="32">
+    <mergeCell ref="B40:H40"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="D10:H10"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B33:H33"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="B32:H32"/>
     <mergeCell ref="D6:H6"/>
+    <mergeCell ref="B41:H41"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B25:H25"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="D7:H7"/>
-    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B21:H21"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:H9"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B14:H14"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B21:H22"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B28:H28"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1206,15 +1386,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.7578125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14.76" customWidth="1" style="44" min="1" max="1"/>
     <col width="38.6" customWidth="1" style="21" min="2" max="2"/>
-    <col width="15.89" customWidth="1" style="44" min="3" max="3"/>
-    <col width="20.43" customWidth="1" style="45" min="4" max="4"/>
-    <col width="15.89" customWidth="1" style="45" min="5" max="5"/>
-    <col width="28.38" customWidth="1" style="45" min="6" max="6"/>
+    <col width="20.43" customWidth="1" style="45" min="3" max="3"/>
+    <col width="15.89" customWidth="1" style="45" min="4" max="4"/>
+    <col width="28.38" customWidth="1" style="45" min="5" max="5"/>
+    <col width="15.89" customWidth="1" style="22" min="6" max="6"/>
+    <col width="34.06" customWidth="1" style="22" min="7" max="7"/>
+    <col hidden="1" width="15.89" customWidth="1" style="44" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1" s="22">
@@ -1230,832 +1412,1044 @@
       </c>
       <c r="C1" s="47" t="inlineStr">
         <is>
+          <t>NISN</t>
+        </is>
+      </c>
+      <c r="D1" s="47" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="E1" s="48" t="inlineStr">
+        <is>
+          <t>NOMOR WALI</t>
+        </is>
+      </c>
+      <c r="F1" s="48" t="inlineStr">
+        <is>
+          <t>JENJANG</t>
+        </is>
+      </c>
+      <c r="G1" s="48" t="inlineStr">
+        <is>
+          <t>NAMA KELAS</t>
+        </is>
+      </c>
+      <c r="H1" s="47" t="inlineStr">
+        <is>
           <t>ID KELAS</t>
-        </is>
-      </c>
-      <c r="D1" s="47" t="inlineStr">
-        <is>
-          <t>NISN</t>
-        </is>
-      </c>
-      <c r="E1" s="47" t="inlineStr">
-        <is>
-          <t>STATUS</t>
-        </is>
-      </c>
-      <c r="F1" s="48" t="inlineStr">
-        <is>
-          <t>NOMOR WALI</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="22">
       <c r="A2" s="49" t="n"/>
       <c r="B2" s="50" t="n"/>
-      <c r="C2" s="51" t="n"/>
+      <c r="C2" s="52" t="n"/>
       <c r="D2" s="52" t="n"/>
       <c r="E2" s="52" t="n"/>
-      <c r="F2" s="52" t="n"/>
+      <c r="F2" s="54" t="n"/>
+      <c r="G2" s="55" t="n"/>
+      <c r="H2" s="51" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="49" t="n"/>
       <c r="B3" s="50" t="n"/>
-      <c r="C3" s="51" t="n"/>
+      <c r="C3" s="52" t="n"/>
       <c r="D3" s="52" t="n"/>
       <c r="E3" s="52" t="n"/>
       <c r="F3" s="52" t="n"/>
+      <c r="G3" s="52" t="n"/>
+      <c r="H3" s="51" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="49" t="n"/>
       <c r="B4" s="50" t="n"/>
-      <c r="C4" s="51" t="n"/>
+      <c r="C4" s="52" t="n"/>
       <c r="D4" s="52" t="n"/>
       <c r="E4" s="52" t="n"/>
       <c r="F4" s="52" t="n"/>
+      <c r="G4" s="52" t="n"/>
+      <c r="H4" s="51" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="49" t="n"/>
       <c r="B5" s="50" t="n"/>
-      <c r="C5" s="51" t="n"/>
+      <c r="C5" s="52" t="n"/>
       <c r="D5" s="52" t="n"/>
       <c r="E5" s="52" t="n"/>
       <c r="F5" s="52" t="n"/>
+      <c r="G5" s="52" t="n"/>
+      <c r="H5" s="51" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="49" t="n"/>
       <c r="B6" s="50" t="n"/>
-      <c r="C6" s="51" t="n"/>
+      <c r="C6" s="52" t="n"/>
       <c r="D6" s="52" t="n"/>
       <c r="E6" s="52" t="n"/>
       <c r="F6" s="52" t="n"/>
+      <c r="G6" s="52" t="n"/>
+      <c r="H6" s="51" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="49" t="n"/>
       <c r="B7" s="50" t="n"/>
-      <c r="C7" s="51" t="n"/>
+      <c r="C7" s="52" t="n"/>
       <c r="D7" s="52" t="n"/>
       <c r="E7" s="52" t="n"/>
       <c r="F7" s="52" t="n"/>
+      <c r="G7" s="52" t="n"/>
+      <c r="H7" s="51" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="49" t="n"/>
       <c r="B8" s="50" t="n"/>
-      <c r="C8" s="51" t="n"/>
+      <c r="C8" s="52" t="n"/>
       <c r="D8" s="52" t="n"/>
       <c r="E8" s="52" t="n"/>
       <c r="F8" s="52" t="n"/>
+      <c r="G8" s="52" t="n"/>
+      <c r="H8" s="51" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="49" t="n"/>
       <c r="B9" s="50" t="n"/>
-      <c r="C9" s="51" t="n"/>
+      <c r="C9" s="52" t="n"/>
       <c r="D9" s="52" t="n"/>
       <c r="E9" s="52" t="n"/>
       <c r="F9" s="52" t="n"/>
+      <c r="G9" s="52" t="n"/>
+      <c r="H9" s="51" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="49" t="n"/>
       <c r="B10" s="50" t="n"/>
-      <c r="C10" s="51" t="n"/>
+      <c r="C10" s="52" t="n"/>
       <c r="D10" s="52" t="n"/>
       <c r="E10" s="52" t="n"/>
       <c r="F10" s="52" t="n"/>
+      <c r="G10" s="52" t="n"/>
+      <c r="H10" s="51" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="49" t="n"/>
       <c r="B11" s="50" t="n"/>
-      <c r="C11" s="51" t="n"/>
+      <c r="C11" s="52" t="n"/>
       <c r="D11" s="52" t="n"/>
       <c r="E11" s="52" t="n"/>
       <c r="F11" s="52" t="n"/>
+      <c r="G11" s="52" t="n"/>
+      <c r="H11" s="51" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="49" t="n"/>
       <c r="B12" s="50" t="n"/>
-      <c r="C12" s="51" t="n"/>
+      <c r="C12" s="52" t="n"/>
       <c r="D12" s="52" t="n"/>
       <c r="E12" s="52" t="n"/>
       <c r="F12" s="52" t="n"/>
+      <c r="G12" s="52" t="n"/>
+      <c r="H12" s="51" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="49" t="n"/>
       <c r="B13" s="50" t="n"/>
-      <c r="C13" s="51" t="n"/>
+      <c r="C13" s="52" t="n"/>
       <c r="D13" s="52" t="n"/>
       <c r="E13" s="52" t="n"/>
       <c r="F13" s="52" t="n"/>
+      <c r="G13" s="52" t="n"/>
+      <c r="H13" s="51" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="49" t="n"/>
       <c r="B14" s="50" t="n"/>
-      <c r="C14" s="51" t="n"/>
+      <c r="C14" s="52" t="n"/>
       <c r="D14" s="52" t="n"/>
       <c r="E14" s="52" t="n"/>
       <c r="F14" s="52" t="n"/>
+      <c r="G14" s="52" t="n"/>
+      <c r="H14" s="51" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="49" t="n"/>
       <c r="B15" s="50" t="n"/>
-      <c r="C15" s="51" t="n"/>
+      <c r="C15" s="52" t="n"/>
       <c r="D15" s="52" t="n"/>
       <c r="E15" s="52" t="n"/>
       <c r="F15" s="52" t="n"/>
+      <c r="G15" s="52" t="n"/>
+      <c r="H15" s="51" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="49" t="n"/>
       <c r="B16" s="50" t="n"/>
-      <c r="C16" s="51" t="n"/>
+      <c r="C16" s="52" t="n"/>
       <c r="D16" s="52" t="n"/>
       <c r="E16" s="52" t="n"/>
       <c r="F16" s="52" t="n"/>
+      <c r="G16" s="52" t="n"/>
+      <c r="H16" s="51" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="49" t="n"/>
       <c r="B17" s="50" t="n"/>
-      <c r="C17" s="51" t="n"/>
+      <c r="C17" s="52" t="n"/>
       <c r="D17" s="52" t="n"/>
       <c r="E17" s="52" t="n"/>
       <c r="F17" s="52" t="n"/>
+      <c r="G17" s="52" t="n"/>
+      <c r="H17" s="51" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="49" t="n"/>
       <c r="B18" s="50" t="n"/>
-      <c r="C18" s="51" t="n"/>
+      <c r="C18" s="52" t="n"/>
       <c r="D18" s="52" t="n"/>
       <c r="E18" s="52" t="n"/>
       <c r="F18" s="52" t="n"/>
+      <c r="G18" s="52" t="n"/>
+      <c r="H18" s="51" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="49" t="n"/>
       <c r="B19" s="50" t="n"/>
-      <c r="C19" s="51" t="n"/>
+      <c r="C19" s="52" t="n"/>
       <c r="D19" s="52" t="n"/>
       <c r="E19" s="52" t="n"/>
       <c r="F19" s="52" t="n"/>
+      <c r="G19" s="52" t="n"/>
+      <c r="H19" s="51" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="49" t="n"/>
       <c r="B20" s="50" t="n"/>
-      <c r="C20" s="51" t="n"/>
+      <c r="C20" s="52" t="n"/>
       <c r="D20" s="52" t="n"/>
       <c r="E20" s="52" t="n"/>
       <c r="F20" s="52" t="n"/>
+      <c r="G20" s="52" t="n"/>
+      <c r="H20" s="51" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="49" t="n"/>
       <c r="B21" s="50" t="n"/>
-      <c r="C21" s="51" t="n"/>
+      <c r="C21" s="52" t="n"/>
       <c r="D21" s="52" t="n"/>
       <c r="E21" s="52" t="n"/>
       <c r="F21" s="52" t="n"/>
+      <c r="G21" s="52" t="n"/>
+      <c r="H21" s="51" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="49" t="n"/>
       <c r="B22" s="50" t="n"/>
-      <c r="C22" s="51" t="n"/>
+      <c r="C22" s="52" t="n"/>
       <c r="D22" s="52" t="n"/>
       <c r="E22" s="52" t="n"/>
       <c r="F22" s="52" t="n"/>
+      <c r="G22" s="52" t="n"/>
+      <c r="H22" s="51" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="49" t="n"/>
       <c r="B23" s="50" t="n"/>
-      <c r="C23" s="51" t="n"/>
+      <c r="C23" s="52" t="n"/>
       <c r="D23" s="52" t="n"/>
       <c r="E23" s="52" t="n"/>
       <c r="F23" s="52" t="n"/>
+      <c r="G23" s="52" t="n"/>
+      <c r="H23" s="51" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="49" t="n"/>
       <c r="B24" s="50" t="n"/>
-      <c r="C24" s="51" t="n"/>
+      <c r="C24" s="52" t="n"/>
       <c r="D24" s="52" t="n"/>
       <c r="E24" s="52" t="n"/>
       <c r="F24" s="52" t="n"/>
+      <c r="G24" s="52" t="n"/>
+      <c r="H24" s="51" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="49" t="n"/>
       <c r="B25" s="50" t="n"/>
-      <c r="C25" s="51" t="n"/>
+      <c r="C25" s="52" t="n"/>
       <c r="D25" s="52" t="n"/>
       <c r="E25" s="52" t="n"/>
       <c r="F25" s="52" t="n"/>
+      <c r="G25" s="52" t="n"/>
+      <c r="H25" s="51" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="49" t="n"/>
       <c r="B26" s="50" t="n"/>
-      <c r="C26" s="51" t="n"/>
+      <c r="C26" s="52" t="n"/>
       <c r="D26" s="52" t="n"/>
       <c r="E26" s="52" t="n"/>
       <c r="F26" s="52" t="n"/>
+      <c r="G26" s="52" t="n"/>
+      <c r="H26" s="51" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="49" t="n"/>
       <c r="B27" s="50" t="n"/>
-      <c r="C27" s="51" t="n"/>
+      <c r="C27" s="52" t="n"/>
       <c r="D27" s="52" t="n"/>
       <c r="E27" s="52" t="n"/>
       <c r="F27" s="52" t="n"/>
+      <c r="G27" s="52" t="n"/>
+      <c r="H27" s="51" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="49" t="n"/>
       <c r="B28" s="50" t="n"/>
-      <c r="C28" s="51" t="n"/>
+      <c r="C28" s="52" t="n"/>
       <c r="D28" s="52" t="n"/>
       <c r="E28" s="52" t="n"/>
       <c r="F28" s="52" t="n"/>
+      <c r="G28" s="52" t="n"/>
+      <c r="H28" s="51" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="49" t="n"/>
       <c r="B29" s="50" t="n"/>
-      <c r="C29" s="51" t="n"/>
+      <c r="C29" s="52" t="n"/>
       <c r="D29" s="52" t="n"/>
       <c r="E29" s="52" t="n"/>
       <c r="F29" s="52" t="n"/>
+      <c r="G29" s="52" t="n"/>
+      <c r="H29" s="51" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="49" t="n"/>
       <c r="B30" s="50" t="n"/>
-      <c r="C30" s="51" t="n"/>
+      <c r="C30" s="52" t="n"/>
       <c r="D30" s="52" t="n"/>
       <c r="E30" s="52" t="n"/>
       <c r="F30" s="52" t="n"/>
+      <c r="G30" s="52" t="n"/>
+      <c r="H30" s="51" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="49" t="n"/>
       <c r="B31" s="50" t="n"/>
-      <c r="C31" s="51" t="n"/>
+      <c r="C31" s="52" t="n"/>
       <c r="D31" s="52" t="n"/>
       <c r="E31" s="52" t="n"/>
       <c r="F31" s="52" t="n"/>
+      <c r="G31" s="52" t="n"/>
+      <c r="H31" s="51" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="49" t="n"/>
       <c r="B32" s="50" t="n"/>
-      <c r="C32" s="51" t="n"/>
+      <c r="C32" s="52" t="n"/>
       <c r="D32" s="52" t="n"/>
       <c r="E32" s="52" t="n"/>
       <c r="F32" s="52" t="n"/>
+      <c r="G32" s="52" t="n"/>
+      <c r="H32" s="51" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="49" t="n"/>
       <c r="B33" s="50" t="n"/>
-      <c r="C33" s="51" t="n"/>
+      <c r="C33" s="52" t="n"/>
       <c r="D33" s="52" t="n"/>
       <c r="E33" s="52" t="n"/>
       <c r="F33" s="52" t="n"/>
+      <c r="G33" s="52" t="n"/>
+      <c r="H33" s="51" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="49" t="n"/>
       <c r="B34" s="50" t="n"/>
-      <c r="C34" s="51" t="n"/>
+      <c r="C34" s="52" t="n"/>
       <c r="D34" s="52" t="n"/>
       <c r="E34" s="52" t="n"/>
       <c r="F34" s="52" t="n"/>
+      <c r="G34" s="52" t="n"/>
+      <c r="H34" s="51" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="49" t="n"/>
       <c r="B35" s="50" t="n"/>
-      <c r="C35" s="51" t="n"/>
+      <c r="C35" s="52" t="n"/>
       <c r="D35" s="52" t="n"/>
       <c r="E35" s="52" t="n"/>
       <c r="F35" s="52" t="n"/>
+      <c r="G35" s="52" t="n"/>
+      <c r="H35" s="51" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="49" t="n"/>
       <c r="B36" s="50" t="n"/>
-      <c r="C36" s="51" t="n"/>
+      <c r="C36" s="52" t="n"/>
       <c r="D36" s="52" t="n"/>
       <c r="E36" s="52" t="n"/>
       <c r="F36" s="52" t="n"/>
+      <c r="G36" s="52" t="n"/>
+      <c r="H36" s="51" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="49" t="n"/>
       <c r="B37" s="50" t="n"/>
-      <c r="C37" s="51" t="n"/>
+      <c r="C37" s="52" t="n"/>
       <c r="D37" s="52" t="n"/>
       <c r="E37" s="52" t="n"/>
       <c r="F37" s="52" t="n"/>
+      <c r="G37" s="52" t="n"/>
+      <c r="H37" s="51" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="49" t="n"/>
       <c r="B38" s="50" t="n"/>
-      <c r="C38" s="51" t="n"/>
+      <c r="C38" s="52" t="n"/>
       <c r="D38" s="52" t="n"/>
       <c r="E38" s="52" t="n"/>
       <c r="F38" s="52" t="n"/>
+      <c r="G38" s="52" t="n"/>
+      <c r="H38" s="51" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="49" t="n"/>
       <c r="B39" s="50" t="n"/>
-      <c r="C39" s="51" t="n"/>
+      <c r="C39" s="52" t="n"/>
       <c r="D39" s="52" t="n"/>
       <c r="E39" s="52" t="n"/>
       <c r="F39" s="52" t="n"/>
+      <c r="G39" s="52" t="n"/>
+      <c r="H39" s="51" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="49" t="n"/>
       <c r="B40" s="50" t="n"/>
-      <c r="C40" s="51" t="n"/>
+      <c r="C40" s="52" t="n"/>
       <c r="D40" s="52" t="n"/>
       <c r="E40" s="52" t="n"/>
       <c r="F40" s="52" t="n"/>
+      <c r="G40" s="52" t="n"/>
+      <c r="H40" s="51" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="49" t="n"/>
       <c r="B41" s="50" t="n"/>
-      <c r="C41" s="51" t="n"/>
+      <c r="C41" s="52" t="n"/>
       <c r="D41" s="52" t="n"/>
       <c r="E41" s="52" t="n"/>
       <c r="F41" s="52" t="n"/>
+      <c r="G41" s="52" t="n"/>
+      <c r="H41" s="51" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="49" t="n"/>
       <c r="B42" s="50" t="n"/>
-      <c r="C42" s="51" t="n"/>
+      <c r="C42" s="52" t="n"/>
       <c r="D42" s="52" t="n"/>
       <c r="E42" s="52" t="n"/>
       <c r="F42" s="52" t="n"/>
+      <c r="G42" s="52" t="n"/>
+      <c r="H42" s="51" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="49" t="n"/>
       <c r="B43" s="50" t="n"/>
-      <c r="C43" s="51" t="n"/>
+      <c r="C43" s="52" t="n"/>
       <c r="D43" s="52" t="n"/>
       <c r="E43" s="52" t="n"/>
       <c r="F43" s="52" t="n"/>
+      <c r="G43" s="52" t="n"/>
+      <c r="H43" s="51" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="49" t="n"/>
       <c r="B44" s="50" t="n"/>
-      <c r="C44" s="51" t="n"/>
+      <c r="C44" s="52" t="n"/>
       <c r="D44" s="52" t="n"/>
       <c r="E44" s="52" t="n"/>
       <c r="F44" s="52" t="n"/>
+      <c r="G44" s="52" t="n"/>
+      <c r="H44" s="51" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="49" t="n"/>
       <c r="B45" s="50" t="n"/>
-      <c r="C45" s="51" t="n"/>
+      <c r="C45" s="52" t="n"/>
       <c r="D45" s="52" t="n"/>
       <c r="E45" s="52" t="n"/>
       <c r="F45" s="52" t="n"/>
+      <c r="G45" s="52" t="n"/>
+      <c r="H45" s="51" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="49" t="n"/>
       <c r="B46" s="50" t="n"/>
-      <c r="C46" s="51" t="n"/>
+      <c r="C46" s="52" t="n"/>
       <c r="D46" s="52" t="n"/>
       <c r="E46" s="52" t="n"/>
       <c r="F46" s="52" t="n"/>
+      <c r="G46" s="52" t="n"/>
+      <c r="H46" s="51" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="49" t="n"/>
       <c r="B47" s="50" t="n"/>
-      <c r="C47" s="51" t="n"/>
+      <c r="C47" s="52" t="n"/>
       <c r="D47" s="52" t="n"/>
       <c r="E47" s="52" t="n"/>
       <c r="F47" s="52" t="n"/>
+      <c r="G47" s="52" t="n"/>
+      <c r="H47" s="51" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="49" t="n"/>
       <c r="B48" s="50" t="n"/>
-      <c r="C48" s="51" t="n"/>
+      <c r="C48" s="52" t="n"/>
       <c r="D48" s="52" t="n"/>
       <c r="E48" s="52" t="n"/>
       <c r="F48" s="52" t="n"/>
+      <c r="G48" s="52" t="n"/>
+      <c r="H48" s="51" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="49" t="n"/>
       <c r="B49" s="50" t="n"/>
-      <c r="C49" s="51" t="n"/>
+      <c r="C49" s="52" t="n"/>
       <c r="D49" s="52" t="n"/>
       <c r="E49" s="52" t="n"/>
       <c r="F49" s="52" t="n"/>
+      <c r="G49" s="52" t="n"/>
+      <c r="H49" s="51" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="49" t="n"/>
       <c r="B50" s="50" t="n"/>
-      <c r="C50" s="51" t="n"/>
+      <c r="C50" s="52" t="n"/>
       <c r="D50" s="52" t="n"/>
       <c r="E50" s="52" t="n"/>
       <c r="F50" s="52" t="n"/>
+      <c r="G50" s="52" t="n"/>
+      <c r="H50" s="51" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="49" t="n"/>
       <c r="B51" s="50" t="n"/>
-      <c r="C51" s="51" t="n"/>
+      <c r="C51" s="52" t="n"/>
       <c r="D51" s="52" t="n"/>
       <c r="E51" s="52" t="n"/>
       <c r="F51" s="52" t="n"/>
+      <c r="G51" s="52" t="n"/>
+      <c r="H51" s="51" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="49" t="n"/>
       <c r="B52" s="50" t="n"/>
-      <c r="C52" s="51" t="n"/>
+      <c r="C52" s="52" t="n"/>
       <c r="D52" s="52" t="n"/>
       <c r="E52" s="52" t="n"/>
       <c r="F52" s="52" t="n"/>
+      <c r="G52" s="52" t="n"/>
+      <c r="H52" s="51" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="49" t="n"/>
       <c r="B53" s="50" t="n"/>
-      <c r="C53" s="51" t="n"/>
+      <c r="C53" s="52" t="n"/>
       <c r="D53" s="52" t="n"/>
       <c r="E53" s="52" t="n"/>
       <c r="F53" s="52" t="n"/>
+      <c r="G53" s="52" t="n"/>
+      <c r="H53" s="51" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="49" t="n"/>
       <c r="B54" s="50" t="n"/>
-      <c r="C54" s="51" t="n"/>
+      <c r="C54" s="52" t="n"/>
       <c r="D54" s="52" t="n"/>
       <c r="E54" s="52" t="n"/>
       <c r="F54" s="52" t="n"/>
+      <c r="G54" s="52" t="n"/>
+      <c r="H54" s="51" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="49" t="n"/>
       <c r="B55" s="50" t="n"/>
-      <c r="C55" s="51" t="n"/>
+      <c r="C55" s="52" t="n"/>
       <c r="D55" s="52" t="n"/>
       <c r="E55" s="52" t="n"/>
       <c r="F55" s="52" t="n"/>
+      <c r="G55" s="52" t="n"/>
+      <c r="H55" s="51" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="49" t="n"/>
       <c r="B56" s="50" t="n"/>
-      <c r="C56" s="51" t="n"/>
+      <c r="C56" s="52" t="n"/>
       <c r="D56" s="52" t="n"/>
       <c r="E56" s="52" t="n"/>
       <c r="F56" s="52" t="n"/>
+      <c r="G56" s="52" t="n"/>
+      <c r="H56" s="51" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="49" t="n"/>
       <c r="B57" s="50" t="n"/>
-      <c r="C57" s="51" t="n"/>
+      <c r="C57" s="52" t="n"/>
       <c r="D57" s="52" t="n"/>
       <c r="E57" s="52" t="n"/>
       <c r="F57" s="52" t="n"/>
+      <c r="G57" s="52" t="n"/>
+      <c r="H57" s="51" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="49" t="n"/>
       <c r="B58" s="50" t="n"/>
-      <c r="C58" s="51" t="n"/>
+      <c r="C58" s="52" t="n"/>
       <c r="D58" s="52" t="n"/>
       <c r="E58" s="52" t="n"/>
       <c r="F58" s="52" t="n"/>
+      <c r="G58" s="52" t="n"/>
+      <c r="H58" s="51" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="49" t="n"/>
       <c r="B59" s="50" t="n"/>
-      <c r="C59" s="51" t="n"/>
+      <c r="C59" s="52" t="n"/>
       <c r="D59" s="52" t="n"/>
       <c r="E59" s="52" t="n"/>
       <c r="F59" s="52" t="n"/>
+      <c r="G59" s="52" t="n"/>
+      <c r="H59" s="51" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="49" t="n"/>
       <c r="B60" s="50" t="n"/>
-      <c r="C60" s="51" t="n"/>
+      <c r="C60" s="52" t="n"/>
       <c r="D60" s="52" t="n"/>
       <c r="E60" s="52" t="n"/>
       <c r="F60" s="52" t="n"/>
+      <c r="G60" s="52" t="n"/>
+      <c r="H60" s="51" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="49" t="n"/>
       <c r="B61" s="50" t="n"/>
-      <c r="C61" s="51" t="n"/>
+      <c r="C61" s="52" t="n"/>
       <c r="D61" s="52" t="n"/>
       <c r="E61" s="52" t="n"/>
       <c r="F61" s="52" t="n"/>
+      <c r="G61" s="52" t="n"/>
+      <c r="H61" s="51" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="49" t="n"/>
       <c r="B62" s="50" t="n"/>
-      <c r="C62" s="51" t="n"/>
+      <c r="C62" s="52" t="n"/>
       <c r="D62" s="52" t="n"/>
       <c r="E62" s="52" t="n"/>
       <c r="F62" s="52" t="n"/>
+      <c r="G62" s="52" t="n"/>
+      <c r="H62" s="51" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="49" t="n"/>
       <c r="B63" s="50" t="n"/>
-      <c r="C63" s="51" t="n"/>
+      <c r="C63" s="52" t="n"/>
       <c r="D63" s="52" t="n"/>
       <c r="E63" s="52" t="n"/>
       <c r="F63" s="52" t="n"/>
+      <c r="G63" s="52" t="n"/>
+      <c r="H63" s="51" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="49" t="n"/>
       <c r="B64" s="50" t="n"/>
-      <c r="C64" s="51" t="n"/>
+      <c r="C64" s="52" t="n"/>
       <c r="D64" s="52" t="n"/>
       <c r="E64" s="52" t="n"/>
       <c r="F64" s="52" t="n"/>
+      <c r="G64" s="52" t="n"/>
+      <c r="H64" s="51" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="49" t="n"/>
       <c r="B65" s="50" t="n"/>
-      <c r="C65" s="51" t="n"/>
+      <c r="C65" s="52" t="n"/>
       <c r="D65" s="52" t="n"/>
       <c r="E65" s="52" t="n"/>
       <c r="F65" s="52" t="n"/>
+      <c r="G65" s="52" t="n"/>
+      <c r="H65" s="51" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="49" t="n"/>
       <c r="B66" s="50" t="n"/>
-      <c r="C66" s="51" t="n"/>
+      <c r="C66" s="52" t="n"/>
       <c r="D66" s="52" t="n"/>
       <c r="E66" s="52" t="n"/>
       <c r="F66" s="52" t="n"/>
+      <c r="G66" s="52" t="n"/>
+      <c r="H66" s="51" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="49" t="n"/>
       <c r="B67" s="50" t="n"/>
-      <c r="C67" s="51" t="n"/>
+      <c r="C67" s="52" t="n"/>
       <c r="D67" s="52" t="n"/>
       <c r="E67" s="52" t="n"/>
       <c r="F67" s="52" t="n"/>
+      <c r="G67" s="52" t="n"/>
+      <c r="H67" s="51" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="49" t="n"/>
       <c r="B68" s="50" t="n"/>
-      <c r="C68" s="51" t="n"/>
+      <c r="C68" s="52" t="n"/>
       <c r="D68" s="52" t="n"/>
       <c r="E68" s="52" t="n"/>
       <c r="F68" s="52" t="n"/>
+      <c r="G68" s="52" t="n"/>
+      <c r="H68" s="51" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="49" t="n"/>
       <c r="B69" s="50" t="n"/>
-      <c r="C69" s="51" t="n"/>
+      <c r="C69" s="52" t="n"/>
       <c r="D69" s="52" t="n"/>
       <c r="E69" s="52" t="n"/>
       <c r="F69" s="52" t="n"/>
+      <c r="G69" s="52" t="n"/>
+      <c r="H69" s="51" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="49" t="n"/>
       <c r="B70" s="50" t="n"/>
-      <c r="C70" s="51" t="n"/>
+      <c r="C70" s="52" t="n"/>
       <c r="D70" s="52" t="n"/>
       <c r="E70" s="52" t="n"/>
       <c r="F70" s="52" t="n"/>
+      <c r="G70" s="52" t="n"/>
+      <c r="H70" s="51" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="49" t="n"/>
       <c r="B71" s="50" t="n"/>
-      <c r="C71" s="51" t="n"/>
+      <c r="C71" s="52" t="n"/>
       <c r="D71" s="52" t="n"/>
       <c r="E71" s="52" t="n"/>
       <c r="F71" s="52" t="n"/>
+      <c r="G71" s="52" t="n"/>
+      <c r="H71" s="51" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="49" t="n"/>
       <c r="B72" s="50" t="n"/>
-      <c r="C72" s="51" t="n"/>
+      <c r="C72" s="52" t="n"/>
       <c r="D72" s="52" t="n"/>
       <c r="E72" s="52" t="n"/>
       <c r="F72" s="52" t="n"/>
+      <c r="G72" s="52" t="n"/>
+      <c r="H72" s="51" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="49" t="n"/>
       <c r="B73" s="50" t="n"/>
-      <c r="C73" s="51" t="n"/>
+      <c r="C73" s="52" t="n"/>
       <c r="D73" s="52" t="n"/>
       <c r="E73" s="52" t="n"/>
       <c r="F73" s="52" t="n"/>
+      <c r="G73" s="52" t="n"/>
+      <c r="H73" s="51" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="49" t="n"/>
       <c r="B74" s="50" t="n"/>
-      <c r="C74" s="51" t="n"/>
+      <c r="C74" s="52" t="n"/>
       <c r="D74" s="52" t="n"/>
       <c r="E74" s="52" t="n"/>
       <c r="F74" s="52" t="n"/>
+      <c r="G74" s="52" t="n"/>
+      <c r="H74" s="51" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="49" t="n"/>
       <c r="B75" s="50" t="n"/>
-      <c r="C75" s="51" t="n"/>
+      <c r="C75" s="52" t="n"/>
       <c r="D75" s="52" t="n"/>
       <c r="E75" s="52" t="n"/>
       <c r="F75" s="52" t="n"/>
+      <c r="G75" s="52" t="n"/>
+      <c r="H75" s="51" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="49" t="n"/>
       <c r="B76" s="50" t="n"/>
-      <c r="C76" s="51" t="n"/>
+      <c r="C76" s="52" t="n"/>
       <c r="D76" s="52" t="n"/>
       <c r="E76" s="52" t="n"/>
       <c r="F76" s="52" t="n"/>
+      <c r="G76" s="52" t="n"/>
+      <c r="H76" s="51" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="49" t="n"/>
       <c r="B77" s="50" t="n"/>
-      <c r="C77" s="51" t="n"/>
+      <c r="C77" s="52" t="n"/>
       <c r="D77" s="52" t="n"/>
       <c r="E77" s="52" t="n"/>
       <c r="F77" s="52" t="n"/>
+      <c r="G77" s="52" t="n"/>
+      <c r="H77" s="51" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="49" t="n"/>
       <c r="B78" s="50" t="n"/>
-      <c r="C78" s="51" t="n"/>
+      <c r="C78" s="52" t="n"/>
       <c r="D78" s="52" t="n"/>
       <c r="E78" s="52" t="n"/>
       <c r="F78" s="52" t="n"/>
+      <c r="G78" s="52" t="n"/>
+      <c r="H78" s="51" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="49" t="n"/>
       <c r="B79" s="50" t="n"/>
-      <c r="C79" s="51" t="n"/>
+      <c r="C79" s="52" t="n"/>
       <c r="D79" s="52" t="n"/>
       <c r="E79" s="52" t="n"/>
       <c r="F79" s="52" t="n"/>
+      <c r="G79" s="52" t="n"/>
+      <c r="H79" s="51" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="49" t="n"/>
       <c r="B80" s="50" t="n"/>
-      <c r="C80" s="51" t="n"/>
+      <c r="C80" s="52" t="n"/>
       <c r="D80" s="52" t="n"/>
       <c r="E80" s="52" t="n"/>
       <c r="F80" s="52" t="n"/>
+      <c r="G80" s="52" t="n"/>
+      <c r="H80" s="51" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="49" t="n"/>
       <c r="B81" s="50" t="n"/>
-      <c r="C81" s="51" t="n"/>
+      <c r="C81" s="52" t="n"/>
       <c r="D81" s="52" t="n"/>
       <c r="E81" s="52" t="n"/>
       <c r="F81" s="52" t="n"/>
+      <c r="G81" s="52" t="n"/>
+      <c r="H81" s="51" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="49" t="n"/>
       <c r="B82" s="50" t="n"/>
-      <c r="C82" s="51" t="n"/>
+      <c r="C82" s="52" t="n"/>
       <c r="D82" s="52" t="n"/>
       <c r="E82" s="52" t="n"/>
       <c r="F82" s="52" t="n"/>
+      <c r="G82" s="52" t="n"/>
+      <c r="H82" s="51" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="49" t="n"/>
       <c r="B83" s="50" t="n"/>
-      <c r="C83" s="51" t="n"/>
+      <c r="C83" s="52" t="n"/>
       <c r="D83" s="52" t="n"/>
       <c r="E83" s="52" t="n"/>
       <c r="F83" s="52" t="n"/>
+      <c r="G83" s="52" t="n"/>
+      <c r="H83" s="51" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="49" t="n"/>
       <c r="B84" s="50" t="n"/>
-      <c r="C84" s="51" t="n"/>
+      <c r="C84" s="52" t="n"/>
       <c r="D84" s="52" t="n"/>
       <c r="E84" s="52" t="n"/>
       <c r="F84" s="52" t="n"/>
+      <c r="G84" s="52" t="n"/>
+      <c r="H84" s="51" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="49" t="n"/>
       <c r="B85" s="50" t="n"/>
-      <c r="C85" s="51" t="n"/>
+      <c r="C85" s="52" t="n"/>
       <c r="D85" s="52" t="n"/>
       <c r="E85" s="52" t="n"/>
       <c r="F85" s="52" t="n"/>
+      <c r="G85" s="52" t="n"/>
+      <c r="H85" s="51" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="49" t="n"/>
       <c r="B86" s="50" t="n"/>
-      <c r="C86" s="51" t="n"/>
+      <c r="C86" s="52" t="n"/>
       <c r="D86" s="52" t="n"/>
       <c r="E86" s="52" t="n"/>
       <c r="F86" s="52" t="n"/>
+      <c r="G86" s="52" t="n"/>
+      <c r="H86" s="51" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="49" t="n"/>
       <c r="B87" s="50" t="n"/>
-      <c r="C87" s="51" t="n"/>
+      <c r="C87" s="52" t="n"/>
       <c r="D87" s="52" t="n"/>
       <c r="E87" s="52" t="n"/>
       <c r="F87" s="52" t="n"/>
+      <c r="G87" s="52" t="n"/>
+      <c r="H87" s="51" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="49" t="n"/>
       <c r="B88" s="50" t="n"/>
-      <c r="C88" s="51" t="n"/>
+      <c r="C88" s="52" t="n"/>
       <c r="D88" s="52" t="n"/>
       <c r="E88" s="52" t="n"/>
       <c r="F88" s="52" t="n"/>
+      <c r="G88" s="52" t="n"/>
+      <c r="H88" s="51" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="49" t="n"/>
       <c r="B89" s="50" t="n"/>
-      <c r="C89" s="51" t="n"/>
+      <c r="C89" s="52" t="n"/>
       <c r="D89" s="52" t="n"/>
       <c r="E89" s="52" t="n"/>
       <c r="F89" s="52" t="n"/>
+      <c r="G89" s="52" t="n"/>
+      <c r="H89" s="51" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="49" t="n"/>
       <c r="B90" s="50" t="n"/>
-      <c r="C90" s="51" t="n"/>
+      <c r="C90" s="52" t="n"/>
       <c r="D90" s="52" t="n"/>
       <c r="E90" s="52" t="n"/>
       <c r="F90" s="52" t="n"/>
+      <c r="G90" s="52" t="n"/>
+      <c r="H90" s="51" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="49" t="n"/>
       <c r="B91" s="50" t="n"/>
-      <c r="C91" s="51" t="n"/>
+      <c r="C91" s="52" t="n"/>
       <c r="D91" s="52" t="n"/>
       <c r="E91" s="52" t="n"/>
       <c r="F91" s="52" t="n"/>
+      <c r="G91" s="52" t="n"/>
+      <c r="H91" s="51" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="49" t="n"/>
       <c r="B92" s="50" t="n"/>
-      <c r="C92" s="51" t="n"/>
+      <c r="C92" s="52" t="n"/>
       <c r="D92" s="52" t="n"/>
       <c r="E92" s="52" t="n"/>
       <c r="F92" s="52" t="n"/>
+      <c r="G92" s="52" t="n"/>
+      <c r="H92" s="51" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="49" t="n"/>
       <c r="B93" s="50" t="n"/>
-      <c r="C93" s="51" t="n"/>
+      <c r="C93" s="52" t="n"/>
       <c r="D93" s="52" t="n"/>
       <c r="E93" s="52" t="n"/>
       <c r="F93" s="52" t="n"/>
+      <c r="G93" s="52" t="n"/>
+      <c r="H93" s="51" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="49" t="n"/>
       <c r="B94" s="50" t="n"/>
-      <c r="C94" s="51" t="n"/>
+      <c r="C94" s="52" t="n"/>
       <c r="D94" s="52" t="n"/>
       <c r="E94" s="52" t="n"/>
       <c r="F94" s="52" t="n"/>
+      <c r="G94" s="52" t="n"/>
+      <c r="H94" s="51" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="49" t="n"/>
       <c r="B95" s="50" t="n"/>
-      <c r="C95" s="51" t="n"/>
+      <c r="C95" s="52" t="n"/>
       <c r="D95" s="52" t="n"/>
       <c r="E95" s="52" t="n"/>
       <c r="F95" s="52" t="n"/>
+      <c r="G95" s="52" t="n"/>
+      <c r="H95" s="51" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="49" t="n"/>
       <c r="B96" s="50" t="n"/>
-      <c r="C96" s="51" t="n"/>
+      <c r="C96" s="52" t="n"/>
       <c r="D96" s="52" t="n"/>
       <c r="E96" s="52" t="n"/>
       <c r="F96" s="52" t="n"/>
+      <c r="G96" s="52" t="n"/>
+      <c r="H96" s="51" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="49" t="n"/>
       <c r="B97" s="50" t="n"/>
-      <c r="C97" s="51" t="n"/>
+      <c r="C97" s="52" t="n"/>
       <c r="D97" s="52" t="n"/>
       <c r="E97" s="52" t="n"/>
       <c r="F97" s="52" t="n"/>
+      <c r="G97" s="52" t="n"/>
+      <c r="H97" s="51" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="49" t="n"/>
       <c r="B98" s="50" t="n"/>
-      <c r="C98" s="51" t="n"/>
+      <c r="C98" s="52" t="n"/>
       <c r="D98" s="52" t="n"/>
       <c r="E98" s="52" t="n"/>
       <c r="F98" s="52" t="n"/>
+      <c r="G98" s="52" t="n"/>
+      <c r="H98" s="51" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="49" t="n"/>
       <c r="B99" s="50" t="n"/>
-      <c r="C99" s="51" t="n"/>
+      <c r="C99" s="52" t="n"/>
       <c r="D99" s="52" t="n"/>
       <c r="E99" s="52" t="n"/>
       <c r="F99" s="52" t="n"/>
+      <c r="G99" s="52" t="n"/>
+      <c r="H99" s="51" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="49" t="n"/>
       <c r="B100" s="50" t="n"/>
-      <c r="C100" s="51" t="n"/>
+      <c r="C100" s="52" t="n"/>
       <c r="D100" s="52" t="n"/>
       <c r="E100" s="52" t="n"/>
       <c r="F100" s="52" t="n"/>
+      <c r="G100" s="52" t="n"/>
+      <c r="H100" s="51" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="49" t="n"/>
       <c r="B101" s="50" t="n"/>
-      <c r="C101" s="51" t="n"/>
+      <c r="C101" s="52" t="n"/>
       <c r="D101" s="52" t="n"/>
       <c r="E101" s="52" t="n"/>
       <c r="F101" s="52" t="n"/>
+      <c r="G101" s="52" t="n"/>
+      <c r="H101" s="51" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="49" t="n"/>
       <c r="B102" s="50" t="n"/>
-      <c r="C102" s="51" t="n"/>
+      <c r="C102" s="52" t="n"/>
       <c r="D102" s="52" t="n"/>
       <c r="E102" s="52" t="n"/>
       <c r="F102" s="52" t="n"/>
+      <c r="G102" s="52" t="n"/>
+      <c r="H102" s="51" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -2067,20 +2461,20 @@
       <formula1>1</formula1>
       <formula2>255</formula2>
     </dataValidation>
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." promptTitle="ID kelas" prompt="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." promptTitle="ID kelas" prompt="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik." promptTitle="NISN" prompt="Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik." type="custom" errorStyle="stop" operator="between">
-      <formula1>OR(D2="",AND(LEN(D2)=10,SUMPRODUCT(--ISNUMBER(FIND(MID(D2,ROW($1:$10),1),"0123456789")))=10,COUNTIF($D$2:$D$1048576,D2)=1))</formula1>
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik." promptTitle="NISN" prompt="Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik." type="custom" errorStyle="stop" operator="between">
+      <formula1>OR(C2="",AND(LEN(C2)=10,SUMPRODUCT(--ISNUMBER(FIND(MID(C2,ROW($1:$10),1),"0123456789")))=10,COUNTIF($C$2:$C$1048576,C2)=1))</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Pilih Aktif atau Tidak aktif." promptTitle="Status siswa" prompt="Pilih Aktif atau Tidak aktif." type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Pilih Aktif atau Tidak aktif." promptTitle="Status siswa" prompt="Pilih Aktif atau Tidak aktif." type="list" errorStyle="stop" operator="between">
       <formula1>"Aktif,Tidak aktif"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit." promptTitle="Nomor wali" prompt="Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit." type="custom" errorStyle="stop">
-      <formula1>OR(F2="",AND(LEN(F2)&lt;=32,OR(LEFT(F2,2)="08",LEFT(F2,3)="628"),SUMPRODUCT(--ISNUMBER(FIND(MID(F2,ROW($1:$32),1),"0123456789")),--(ROW($1:$32)&lt;=LEN(F2)))=LEN(F2)))</formula1>
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit." promptTitle="Nomor wali" prompt="Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit." type="custom" errorStyle="stop">
+      <formula1>OR(E2="",AND(LEN(E2)&lt;=32,OR(LEFT(E2,2)="08",LEFT(E2,3)="628"),SUMPRODUCT(--ISNUMBER(FIND(MID(E2,ROW($1:$32),1),"0123456789")),--(ROW($1:$32)&lt;=LEN(E2)))=LEN(E2)))</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2091,4 +2485,565 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <tabColor rgb="FFD8EEEE"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:C102"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.7578125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.35" customWidth="1" style="43" min="1" max="1"/>
+    <col width="15.89" customWidth="1" style="43" min="2" max="2"/>
+    <col width="34.06" customWidth="1" style="44" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customFormat="1" customHeight="1" s="21">
+      <c r="A1" s="56" t="inlineStr">
+        <is>
+          <t>ID KELAS</t>
+        </is>
+      </c>
+      <c r="B1" s="57" t="inlineStr">
+        <is>
+          <t>JENJANG</t>
+        </is>
+      </c>
+      <c r="C1" s="58" t="inlineStr">
+        <is>
+          <t>NAMA KELAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customFormat="1" customHeight="1" s="21">
+      <c r="A2" s="59" t="n"/>
+      <c r="B2" s="60" t="n"/>
+      <c r="C2" s="61" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="59" t="n"/>
+      <c r="B3" s="60" t="n"/>
+      <c r="C3" s="61" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="59" t="n"/>
+      <c r="B4" s="60" t="n"/>
+      <c r="C4" s="61" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="59" t="n"/>
+      <c r="B5" s="60" t="n"/>
+      <c r="C5" s="61" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="59" t="n"/>
+      <c r="B6" s="60" t="n"/>
+      <c r="C6" s="61" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="59" t="n"/>
+      <c r="B7" s="60" t="n"/>
+      <c r="C7" s="61" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="59" t="n"/>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="61" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="n"/>
+      <c r="B9" s="60" t="n"/>
+      <c r="C9" s="61" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="59" t="n"/>
+      <c r="B10" s="60" t="n"/>
+      <c r="C10" s="61" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="59" t="n"/>
+      <c r="B11" s="60" t="n"/>
+      <c r="C11" s="61" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="59" t="n"/>
+      <c r="B12" s="60" t="n"/>
+      <c r="C12" s="61" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="59" t="n"/>
+      <c r="B13" s="60" t="n"/>
+      <c r="C13" s="61" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="59" t="n"/>
+      <c r="B14" s="60" t="n"/>
+      <c r="C14" s="61" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="59" t="n"/>
+      <c r="B15" s="60" t="n"/>
+      <c r="C15" s="61" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="59" t="n"/>
+      <c r="B16" s="60" t="n"/>
+      <c r="C16" s="61" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="59" t="n"/>
+      <c r="B17" s="60" t="n"/>
+      <c r="C17" s="61" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="59" t="n"/>
+      <c r="B18" s="60" t="n"/>
+      <c r="C18" s="61" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="59" t="n"/>
+      <c r="B19" s="60" t="n"/>
+      <c r="C19" s="61" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="59" t="n"/>
+      <c r="B20" s="60" t="n"/>
+      <c r="C20" s="61" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="59" t="n"/>
+      <c r="B21" s="60" t="n"/>
+      <c r="C21" s="61" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="59" t="n"/>
+      <c r="B22" s="60" t="n"/>
+      <c r="C22" s="61" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="59" t="n"/>
+      <c r="B23" s="60" t="n"/>
+      <c r="C23" s="61" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="59" t="n"/>
+      <c r="B24" s="60" t="n"/>
+      <c r="C24" s="61" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="59" t="n"/>
+      <c r="B25" s="60" t="n"/>
+      <c r="C25" s="61" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="59" t="n"/>
+      <c r="B26" s="60" t="n"/>
+      <c r="C26" s="61" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="59" t="n"/>
+      <c r="B27" s="60" t="n"/>
+      <c r="C27" s="61" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="59" t="n"/>
+      <c r="B28" s="60" t="n"/>
+      <c r="C28" s="61" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="59" t="n"/>
+      <c r="B29" s="60" t="n"/>
+      <c r="C29" s="61" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="59" t="n"/>
+      <c r="B30" s="60" t="n"/>
+      <c r="C30" s="61" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="59" t="n"/>
+      <c r="B31" s="60" t="n"/>
+      <c r="C31" s="61" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="59" t="n"/>
+      <c r="B32" s="60" t="n"/>
+      <c r="C32" s="61" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="59" t="n"/>
+      <c r="B33" s="60" t="n"/>
+      <c r="C33" s="61" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="59" t="n"/>
+      <c r="B34" s="60" t="n"/>
+      <c r="C34" s="61" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="59" t="n"/>
+      <c r="B35" s="60" t="n"/>
+      <c r="C35" s="61" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="59" t="n"/>
+      <c r="B36" s="60" t="n"/>
+      <c r="C36" s="61" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="59" t="n"/>
+      <c r="B37" s="60" t="n"/>
+      <c r="C37" s="61" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="59" t="n"/>
+      <c r="B38" s="60" t="n"/>
+      <c r="C38" s="61" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="59" t="n"/>
+      <c r="B39" s="60" t="n"/>
+      <c r="C39" s="61" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="59" t="n"/>
+      <c r="B40" s="60" t="n"/>
+      <c r="C40" s="61" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="59" t="n"/>
+      <c r="B41" s="60" t="n"/>
+      <c r="C41" s="61" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="59" t="n"/>
+      <c r="B42" s="60" t="n"/>
+      <c r="C42" s="61" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="59" t="n"/>
+      <c r="B43" s="60" t="n"/>
+      <c r="C43" s="61" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="n"/>
+      <c r="B44" s="60" t="n"/>
+      <c r="C44" s="61" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="59" t="n"/>
+      <c r="B45" s="60" t="n"/>
+      <c r="C45" s="61" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="59" t="n"/>
+      <c r="B46" s="60" t="n"/>
+      <c r="C46" s="61" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="59" t="n"/>
+      <c r="B47" s="60" t="n"/>
+      <c r="C47" s="61" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="59" t="n"/>
+      <c r="B48" s="60" t="n"/>
+      <c r="C48" s="61" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="59" t="n"/>
+      <c r="B49" s="60" t="n"/>
+      <c r="C49" s="61" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="59" t="n"/>
+      <c r="B50" s="60" t="n"/>
+      <c r="C50" s="61" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="59" t="n"/>
+      <c r="B51" s="60" t="n"/>
+      <c r="C51" s="61" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="59" t="n"/>
+      <c r="B52" s="60" t="n"/>
+      <c r="C52" s="61" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="59" t="n"/>
+      <c r="B53" s="60" t="n"/>
+      <c r="C53" s="61" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="59" t="n"/>
+      <c r="B54" s="60" t="n"/>
+      <c r="C54" s="61" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="59" t="n"/>
+      <c r="B55" s="60" t="n"/>
+      <c r="C55" s="61" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="59" t="n"/>
+      <c r="B56" s="60" t="n"/>
+      <c r="C56" s="61" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="59" t="n"/>
+      <c r="B57" s="60" t="n"/>
+      <c r="C57" s="61" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="59" t="n"/>
+      <c r="B58" s="60" t="n"/>
+      <c r="C58" s="61" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="59" t="n"/>
+      <c r="B59" s="60" t="n"/>
+      <c r="C59" s="61" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="59" t="n"/>
+      <c r="B60" s="60" t="n"/>
+      <c r="C60" s="61" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="59" t="n"/>
+      <c r="B61" s="60" t="n"/>
+      <c r="C61" s="61" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="59" t="n"/>
+      <c r="B62" s="60" t="n"/>
+      <c r="C62" s="61" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="59" t="n"/>
+      <c r="B63" s="60" t="n"/>
+      <c r="C63" s="61" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="59" t="n"/>
+      <c r="B64" s="60" t="n"/>
+      <c r="C64" s="61" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="59" t="n"/>
+      <c r="B65" s="60" t="n"/>
+      <c r="C65" s="61" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="59" t="n"/>
+      <c r="B66" s="60" t="n"/>
+      <c r="C66" s="61" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="59" t="n"/>
+      <c r="B67" s="60" t="n"/>
+      <c r="C67" s="61" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="59" t="n"/>
+      <c r="B68" s="60" t="n"/>
+      <c r="C68" s="61" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="59" t="n"/>
+      <c r="B69" s="60" t="n"/>
+      <c r="C69" s="61" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="59" t="n"/>
+      <c r="B70" s="60" t="n"/>
+      <c r="C70" s="61" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="59" t="n"/>
+      <c r="B71" s="60" t="n"/>
+      <c r="C71" s="61" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="59" t="n"/>
+      <c r="B72" s="60" t="n"/>
+      <c r="C72" s="61" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="59" t="n"/>
+      <c r="B73" s="60" t="n"/>
+      <c r="C73" s="61" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="59" t="n"/>
+      <c r="B74" s="60" t="n"/>
+      <c r="C74" s="61" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="59" t="n"/>
+      <c r="B75" s="60" t="n"/>
+      <c r="C75" s="61" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="59" t="n"/>
+      <c r="B76" s="60" t="n"/>
+      <c r="C76" s="61" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="59" t="n"/>
+      <c r="B77" s="60" t="n"/>
+      <c r="C77" s="61" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="59" t="n"/>
+      <c r="B78" s="60" t="n"/>
+      <c r="C78" s="61" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="59" t="n"/>
+      <c r="B79" s="60" t="n"/>
+      <c r="C79" s="61" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="59" t="n"/>
+      <c r="B80" s="60" t="n"/>
+      <c r="C80" s="61" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="59" t="n"/>
+      <c r="B81" s="60" t="n"/>
+      <c r="C81" s="61" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="59" t="n"/>
+      <c r="B82" s="60" t="n"/>
+      <c r="C82" s="61" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="59" t="n"/>
+      <c r="B83" s="60" t="n"/>
+      <c r="C83" s="61" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="59" t="n"/>
+      <c r="B84" s="60" t="n"/>
+      <c r="C84" s="61" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="59" t="n"/>
+      <c r="B85" s="60" t="n"/>
+      <c r="C85" s="61" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="59" t="n"/>
+      <c r="B86" s="60" t="n"/>
+      <c r="C86" s="61" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="59" t="n"/>
+      <c r="B87" s="60" t="n"/>
+      <c r="C87" s="61" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="59" t="n"/>
+      <c r="B88" s="60" t="n"/>
+      <c r="C88" s="61" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="59" t="n"/>
+      <c r="B89" s="60" t="n"/>
+      <c r="C89" s="61" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="59" t="n"/>
+      <c r="B90" s="60" t="n"/>
+      <c r="C90" s="61" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="59" t="n"/>
+      <c r="B91" s="60" t="n"/>
+      <c r="C91" s="61" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="59" t="n"/>
+      <c r="B92" s="60" t="n"/>
+      <c r="C92" s="61" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="59" t="n"/>
+      <c r="B93" s="60" t="n"/>
+      <c r="C93" s="61" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="59" t="n"/>
+      <c r="B94" s="60" t="n"/>
+      <c r="C94" s="61" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="59" t="n"/>
+      <c r="B95" s="60" t="n"/>
+      <c r="C95" s="61" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="59" t="n"/>
+      <c r="B96" s="60" t="n"/>
+      <c r="C96" s="61" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="59" t="n"/>
+      <c r="B97" s="60" t="n"/>
+      <c r="C97" s="61" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="59" t="n"/>
+      <c r="B98" s="60" t="n"/>
+      <c r="C98" s="61" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="59" t="n"/>
+      <c r="B99" s="60" t="n"/>
+      <c r="C99" s="61" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="59" t="n"/>
+      <c r="B100" s="60" t="n"/>
+      <c r="C100" s="61" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="59" t="n"/>
+      <c r="B101" s="60" t="n"/>
+      <c r="C101" s="61" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="59" t="n"/>
+      <c r="B102" s="60" t="n"/>
+      <c r="C102" s="61" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Kosongkan untuk kelas baru. Pertahankan ID untuk mengedit kelas." promptTitle="ID kelas" prompt="Kosongkan untuk kelas baru. Pertahankan ID untuk mengedit kelas." type="custom" errorStyle="stop" operator="between">
+      <formula1>OR(A2="",AND(ISNUMBER(A2),A2=INT(A2),A2&gt;=1,COUNTIF($A$2:$A$1048576,A2)=1))</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi bilangan bulat antara 1 dan 20." promptTitle="Jenjang" prompt="Isi bilangan bulat antara 1 dan 20." type="whole" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi 1–20 karakter. Kombinasi jenjang dan nama kelas harus unik." promptTitle="Nama kelas" prompt="Isi 1–20 karakter. Kombinasi jenjang dan nama kelas harus unik." type="custom" errorStyle="stop" operator="between">
+      <formula1>OR(C2="",AND(LEN(C2)&gt;=1,LEN(C2)&lt;=20,COUNTIFS($B$2:$B$1048576,B2,$C$2:$C$1048576,C2)=1))</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: more proper documentation in import worksheet
</commit_message>
<xml_diff>
--- a/web/app/spreadsheet_templates/students_export_template.xlsx
+++ b/web/app/spreadsheet_templates/students_export_template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="classes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'instructions'!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'instructions'!$B$2:$H$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -93,6 +93,13 @@
       <family val="0"/>
       <color rgb="FF667370"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="9">
@@ -401,7 +408,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -575,6 +582,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
       <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="6" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -708,22 +754,32 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas.</t>
+        <t>Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Tepat 10 digit. Nol di depan harus dipertahankan. NISN harus unik.</t>
+        <t>Pilih Aktif atau Tidak aktif.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Pilih Aktif atau Tidak aktif.</t>
+        <t>Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Opsional. Angka saja, diawali 08 atau 628; maksimal 32 digit.</t>
+        <t>Ketik ID dari sheet classes, termasuk ID sementara N1, N2, dan seterusnya. Tidak ada dropdown.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Kolom rumus, hanya baca. Nilai mengikuti ID KELAS.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Kolom rumus, hanya baca. Ubah nama kelas pada sheet classes.</t>
       </text>
     </comment>
   </commentList>
@@ -739,9 +795,9 @@
     <tableColumn id="3" name="NISN"/>
     <tableColumn id="4" name="STATUS"/>
     <tableColumn id="5" name="NOMOR WALI"/>
-    <tableColumn id="6" name="JENJANG"/>
-    <tableColumn id="7" name="NAMA KELAS"/>
-    <tableColumn id="8" name="ID KELAS"/>
+    <tableColumn id="6" name="ID KELAS"/>
+    <tableColumn id="7" name="JENJANG"/>
+    <tableColumn id="8" name="NAMA KELAS"/>
   </tableColumns>
 </table>
 </file>
@@ -956,7 +1012,7 @@
       <c r="A2" s="23" t="n"/>
       <c r="B2" s="24" t="inlineStr">
         <is>
-          <t>Ekspor &amp; Impor Siswa dan Kelas</t>
+          <t>Panduan Ekspor dan Impor Siswa</t>
         </is>
       </c>
       <c r="G2" s="25" t="inlineStr">
@@ -976,11 +1032,11 @@
       <c r="G3" s="23" t="n"/>
       <c r="H3" s="23" t="n"/>
     </row>
-    <row r="4" ht="23" customHeight="1" s="22">
+    <row r="4" ht="29" customHeight="1" s="22">
       <c r="A4" s="23" t="n"/>
-      <c r="B4" s="27" t="inlineStr">
-        <is>
-          <t>Tentang file ini</t>
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>Dokumentasi lengkap: https://example.com</t>
         </is>
       </c>
       <c r="C4" s="28" t="n"/>
@@ -992,17 +1048,13 @@
     </row>
     <row r="5" ht="34" customHeight="1" s="22">
       <c r="A5" s="23" t="n"/>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>Workbook ini dibuat oleh Absensa untuk ekspor serta penyuntingan massal dan impor kembali.</t>
-        </is>
-      </c>
+      <c r="B5" s="29" t="n"/>
     </row>
     <row r="6" ht="23" customHeight="1" s="22">
       <c r="A6" s="23" t="n"/>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Filter siswa</t>
         </is>
       </c>
       <c r="C6" s="26" t="n"/>
@@ -1020,11 +1072,11 @@
       <c r="A7" s="23" t="n"/>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Waktu ekspor</t>
+          <t>Waktu dibuat</t>
         </is>
       </c>
       <c r="C7" s="26" t="n"/>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>{{ exported_at }}</t>
         </is>
@@ -1038,11 +1090,11 @@
       <c r="A8" s="23" t="n"/>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Jumlah data</t>
+          <t>Jumlah siswa</t>
         </is>
       </c>
       <c r="C8" s="26" t="n"/>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>{{ row_count }}</t>
         </is>
@@ -1054,75 +1106,56 @@
     </row>
     <row r="9" ht="23" customHeight="1" s="22">
       <c r="A9" s="23" t="n"/>
-      <c r="B9" s="30" t="inlineStr">
-        <is>
-          <t>Sheet data</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="n"/>
-      <c r="D9" s="32" t="inlineStr">
-        <is>
-          <t>students dan classes</t>
-        </is>
-      </c>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="G9" s="28" t="n"/>
-      <c r="H9" s="26" t="n"/>
-    </row>
-    <row r="10" ht="23" customHeight="1" s="22">
+      <c r="B9" s="30" t="n"/>
+      <c r="D9" s="32" t="n"/>
+    </row>
+    <row r="10" ht="25" customHeight="1" s="22">
       <c r="A10" s="23" t="n"/>
-      <c r="B10" s="30" t="inlineStr">
-        <is>
-          <t>Kolom ID</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>ID siswa dan ID KELAS (dilindungi)</t>
-        </is>
-      </c>
+      <c r="B10" s="67" t="inlineStr">
+        <is>
+          <t>Tentang file ini</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="n"/>
+      <c r="D10" s="28" t="n"/>
       <c r="E10" s="28" t="n"/>
       <c r="F10" s="28" t="n"/>
       <c r="G10" s="28" t="n"/>
       <c r="H10" s="26" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="22">
+    <row r="11" ht="72" customHeight="1" s="22">
       <c r="A11" s="23" t="n"/>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="23" t="n"/>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="23" t="n"/>
-      <c r="H11" s="23" t="n"/>
+      <c r="B11" s="68" t="inlineStr">
+        <is>
+          <t>Workbook ini dibuat oleh Absensa untuk mengunduh data siswa dan mengimpor data untuk menambah atau mengedit siswa. Anda bisa mendapatkannya dari template impor atau melalui Ekspor di dashboard Siswa maupun dashboard Kelas. Data siswa pada hasil ekspor mengikuti filter yang dipilih; sheet classes selalu memuat semua kelas.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="24" customHeight="1" s="22">
       <c r="A12" s="23" t="n"/>
-      <c r="B12" s="53" t="inlineStr">
-        <is>
-          <t>Isi workbook</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
-      <c r="G12" s="28" t="n"/>
-      <c r="H12" s="26" t="n"/>
-    </row>
-    <row r="13" ht="62" customHeight="1" s="22">
+      <c r="B12" s="53" t="n"/>
+    </row>
+    <row r="13" ht="25" customHeight="1" s="22">
       <c r="A13" s="23" t="n"/>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>students berisi data siswa sesuai filter ekspor di atas. classes selalu berisi seluruh kelas dari semua jenjang, tanpa mengikuti filter siswa, dan menjadi sumber pilihan dropdown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1" s="22">
+      <c r="B13" s="67" t="inlineStr">
+        <is>
+          <t>Sebelum mengedit</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="28" t="n"/>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="72" customHeight="1" s="22">
       <c r="A14" s="23" t="n"/>
-      <c r="B14" s="29" t="n"/>
+      <c r="B14" s="68" t="inlineStr">
+        <is>
+          <t>Jika ingin mengedit siswa yang sudah ada, sebaiknya mulai dari Ekspor pada dashboard Siswa atau Kelas. Hasil ekspor sudah memuat ID dan data siswa saat ini. Pertahankan nilai pada kolom ID (student_id) agar perubahan masuk ke siswa yang benar, lalu lengkapi nilai yang diperlukan; sel kosong tidak berarti nilai lama akan dipertahankan.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="A15" s="23" t="n"/>
@@ -1134,11 +1167,11 @@
       <c r="G15" s="23" t="n"/>
       <c r="H15" s="23" t="n"/>
     </row>
-    <row r="16" ht="24" customHeight="1" s="22">
+    <row r="16" ht="25" customHeight="1" s="22">
       <c r="A16" s="23" t="n"/>
-      <c r="B16" s="53" t="inlineStr">
-        <is>
-          <t>Jangan mengubah identitas</t>
+      <c r="B16" s="67" t="inlineStr">
+        <is>
+          <t>Menambah siswa baru</t>
         </is>
       </c>
       <c r="C16" s="28" t="n"/>
@@ -1148,11 +1181,11 @@
       <c r="G16" s="28" t="n"/>
       <c r="H16" s="26" t="n"/>
     </row>
-    <row r="17" ht="62" customHeight="1" s="22">
+    <row r="17" ht="57" customHeight="1" s="22">
       <c r="A17" s="23" t="n"/>
-      <c r="B17" s="62" t="inlineStr">
-        <is>
-          <t>Jangan mengganti nama sheet, judul kolom, ID siswa, atau ID kelas yang sudah ada. ID kelas adalah identitas tetap meskipun jenjang/nama kelas berubah. ID siswa dan ID pada classes dilindungi. Pada students, ID KELAS dapat diketik untuk menentukan kelas siswa.</t>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>Untuk siswa baru, biarkan kolom ID (student_id) kosong lalu isi data pada satu baris. NISN harus tepat 10 digit; gunakan format teks agar angka nol di depan tetap ada. Pilih STATUS dari daftar yang tersedia. Isi ID KELAS (class_id) pada sel kosong dengan ID dari sheet classes, termasuk ID sementara seperti N1.</t>
         </is>
       </c>
       <c r="C17" s="63" t="n"/>
@@ -1166,82 +1199,88 @@
       <c r="A18" s="23" t="n"/>
       <c r="B18" s="34" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1" s="22">
+    <row r="19" ht="25" customHeight="1" s="22">
       <c r="A19" s="23" t="n"/>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="23" t="n"/>
-      <c r="H19" s="23" t="n"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" s="22">
+      <c r="B19" s="67" t="inlineStr">
+        <is>
+          <t>Mengedit siswa yang sudah ada</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="28" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
+      <c r="H19" s="26" t="n"/>
+    </row>
+    <row r="20" ht="72" customHeight="1" s="22">
       <c r="A20" s="23" t="n"/>
-      <c r="B20" s="53" t="inlineStr">
-        <is>
-          <t>Menentukan kelas siswa dengan ID</t>
-        </is>
-      </c>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="28" t="n"/>
-      <c r="G20" s="28" t="n"/>
-      <c r="H20" s="26" t="n"/>
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>Jika kolom ID (student_id) berisi ID siswa yang sudah terdaftar, baris itu akan mengubah data siswa tersebut. Jangan mengganti ID yang sudah ada secara tidak sengaja. Spreadsheet dapat memeriksa format, tetapi tidak dapat memastikan ID benar-benar ada di sistem. Absensa memeriksanya kembali saat impor dan akan melaporkan jika ID tidak ditemukan.</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="42" t="n"/>
     </row>
     <row r="21" ht="62" customHeight="1" s="22">
       <c r="A21" s="23" t="n"/>
-      <c r="B21" s="65" t="inlineStr">
-        <is>
-          <t>Ketik ID KELAS dari classes, misalnya 17 atau N2; kolom ini tidak memiliki dropdown. Validasi memeriksa apakah ID tersebut ada. JENJANG dan NAMA KELAS adalah kolom rumus yang dikunci dan diberi tampilan berbeda. Ubah kedua nilai itu hanya pada classes. Siswa baru wajib memiliki kelas; siswa lama boleh dikosongkan ID kelasnya.</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="n"/>
-      <c r="D21" s="41" t="n"/>
-      <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
-      <c r="G21" s="41" t="n"/>
-      <c r="H21" s="42" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" s="22">
+      <c r="B21" s="65" t="n"/>
+    </row>
+    <row r="22" ht="25" customHeight="1" s="22">
       <c r="A22" s="23" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="22">
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>Kelas dan ID sementara</t>
+        </is>
+      </c>
+      <c r="C22" s="28" t="n"/>
+      <c r="D22" s="28" t="n"/>
+      <c r="E22" s="28" t="n"/>
+      <c r="F22" s="28" t="n"/>
+      <c r="G22" s="28" t="n"/>
+      <c r="H22" s="26" t="n"/>
+    </row>
+    <row r="23" ht="84" customHeight="1" s="22">
       <c r="A23" s="23" t="n"/>
-      <c r="B23" s="23" t="n"/>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="23" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="23" t="n"/>
-      <c r="G23" s="23" t="n"/>
-      <c r="H23" s="23" t="n"/>
+      <c r="B23" s="68" t="inlineStr">
+        <is>
+          <t>Isi ID KELAS (class_id) pada sel kosong untuk menentukan kelas siswa. ID kelas yang sudah terisi pada data ekspor dilindungi; sel kosong disediakan untuk pengisian siswa baru. Untuk kelas baru, gunakan baris cadangan di sheet classes yang sudah berisi ID seperti N1, N2, dan seterusnya: isi jenjang serta nama kelas pada baris itu, lalu gunakan ID N yang sama pada siswa baru. Absensa menyelesaikan ID sementara saat impor. Mengubah nama atau jenjang kelas pada baris ber-ID tetap akan memperbarui kelas tersebut.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="24" customHeight="1" s="22">
       <c r="A24" s="23" t="n"/>
-      <c r="B24" s="53" t="inlineStr">
-        <is>
-          <t>Kelas baru: ID sementara yang tetap</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="n"/>
-      <c r="D24" s="28" t="n"/>
-      <c r="E24" s="28" t="n"/>
-      <c r="F24" s="28" t="n"/>
-      <c r="G24" s="28" t="n"/>
-      <c r="H24" s="26" t="n"/>
-    </row>
-    <row r="25" ht="90" customHeight="1" s="22">
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>Absensa menyediakan 100 baris baru dengan ID tetap N1–N100. Isi JENJANG dan NAMA KELAS pada baris tersebut, lalu gunakan ID N itu pada students. ID sudah dialokasikan sebagai nilai tetap, bukan rumus nomor baris, sehingga tidak berubah saat baris lain diedit, dipindah, disisipkan, atau dihapus. Baris cadangan yang belum diisi diabaikan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1" s="22">
-      <c r="B28" s="53" t="inlineStr">
-        <is>
-          <t>Rumus langsung mengikuti perubahan kelas</t>
+      <c r="B24" s="53" t="n"/>
+    </row>
+    <row r="25" ht="25" customHeight="1" s="22">
+      <c r="B25" s="67" t="inlineStr">
+        <is>
+          <t>Sel yang dilindungi dan pilihan isian</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="n"/>
+      <c r="D25" s="28" t="n"/>
+      <c r="E25" s="28" t="n"/>
+      <c r="F25" s="28" t="n"/>
+      <c r="G25" s="28" t="n"/>
+      <c r="H25" s="26" t="n"/>
+    </row>
+    <row r="26" ht="72" customHeight="1" s="22">
+      <c r="B26" s="68" t="inlineStr">
+        <is>
+          <t>Kolom JENJANG dan NAMA KELAS mengikuti ID KELAS (class_id) secara otomatis dan tidak untuk diedit. Ubah informasi kelas pada sheet classes. Proteksi dan daftar pilihan membantu mencegah perubahan yang membuat impor bermasalah. Jangan membuka proteksi, menghapus validasi, mengganti nama sheet atau judul kolom, maupun mengubah susunan workbook jika file akan diimpor kembali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1" s="22">
+      <c r="B28" s="67" t="inlineStr">
+        <is>
+          <t>Jika baris tidak cukup</t>
         </is>
       </c>
       <c r="C28" s="28" t="n"/>
@@ -1251,57 +1290,89 @@
       <c r="G28" s="28" t="n"/>
       <c r="H28" s="26" t="n"/>
     </row>
-    <row r="29" ht="86" customHeight="1" s="22">
-      <c r="B29" s="29" t="inlineStr">
-        <is>
-          <t>Contoh: N1 | 10 | X RPL 1 diubah menjadi N1 | 10 | X RPL A pada classes. Siswa dengan ID KELAS N1 langsung menampilkan nama X RPL A melalui VLOOKUP setelah spreadsheet menghitung ulang. ID tidak berubah. Saat impor, Absensa membuat kelas baru, memperoleh ID database, lalu menghubungkan semua siswa yang memakai N1 ke kelas itu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1" s="22">
-      <c r="B32" s="53" t="inlineStr">
-        <is>
-          <t>Menghapus baris BUKAN menghapus kelas</t>
-        </is>
-      </c>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="28" t="n"/>
-      <c r="F32" s="28" t="n"/>
-      <c r="G32" s="28" t="n"/>
-      <c r="H32" s="26" t="n"/>
+    <row r="29" ht="57" customHeight="1" s="22">
+      <c r="B29" s="68" t="inlineStr">
+        <is>
+          <t>Template biasanya menyediakan sekitar 100 baris siap isi. Jika habis, unduh template baru dari server, atau salin sheet siswa yang masih sesuai lalu lanjutkan pengisian di sheet salinan itu. Sheet salinan boleh diberi nama apa pun. Pertahankan kolom, validasi, dan proteksinya agar tetap dapat dikenali saat impor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="25" customHeight="1" s="22">
+      <c r="B31" s="67" t="inlineStr">
+        <is>
+          <t>Mengimpor beberapa file dengan ZIP</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="n"/>
+      <c r="D31" s="28" t="n"/>
+      <c r="E31" s="28" t="n"/>
+      <c r="F31" s="28" t="n"/>
+      <c r="G31" s="28" t="n"/>
+      <c r="H31" s="26" t="n"/>
+    </row>
+    <row r="32" ht="57" customHeight="1" s="22">
+      <c r="B32" s="70" t="inlineStr">
+        <is>
+          <t>Impor menerima satu file .xlsx atau arsip seperti .zip, .rar, .7z, atau .tar yang berisi satu atau beberapa file .xlsx. Jika data dibagi ke beberapa workbook, masukkan semua file Excel ke dalam satu ZIP lalu unggah ZIP tersebut melalui fitur impor massal.</t>
+        </is>
+      </c>
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="41" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="41" t="n"/>
+      <c r="G32" s="41" t="n"/>
+      <c r="H32" s="42" t="n"/>
     </row>
     <row r="33" ht="62" customHeight="1" s="22">
-      <c r="B33" s="29" t="inlineStr">
-        <is>
-          <t>Menghapus baris kelas hanya menghapusnya dari workbook dan pilihan kelasnya, bukan dari Absensa. Siswa yang masih merujuk kelas tersebut perlu disesuaikan atau baris kelas dikembalikan. Penghapusan kelas dari database dilakukan secara eksplisit melalui halaman/dashboard Kelas.</t>
+      <c r="B33" s="29" t="n"/>
+    </row>
+    <row r="34" ht="25" customHeight="1" s="22">
+      <c r="B34" s="67" t="inlineStr">
+        <is>
+          <t>Menambahkan atau mengganti foto siswa</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="n"/>
+      <c r="D34" s="28" t="n"/>
+      <c r="E34" s="28" t="n"/>
+      <c r="F34" s="28" t="n"/>
+      <c r="G34" s="28" t="n"/>
+      <c r="H34" s="26" t="n"/>
+    </row>
+    <row r="35" ht="72" customHeight="1" s="22">
+      <c r="B35" s="68" t="inlineStr">
+        <is>
+          <t>Foto bersifat opsional. Untuk mengirim foto, masukkan file Excel dan folder bernama persis photos/ ke dalam ZIP. Nama file foto harus memakai NISN 10 digit, misalnya photos/0081234567.jpg. Format yang diterima: .jpg, .jpeg, .png, atau .webp. Foto dicocokkan dengan NISN, bukan student_id, dan dapat dipakai untuk siswa baru maupun yang sudah ada jika data siswanya ikut diimpor.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="22">
-      <c r="B36" s="53" t="inlineStr">
-        <is>
-          <t>Impor bersifat semua-atau-tidak-sama-sekali</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="28" t="n"/>
-      <c r="F36" s="28" t="n"/>
-      <c r="G36" s="28" t="n"/>
-      <c r="H36" s="26" t="n"/>
-    </row>
-    <row r="37" ht="62" customHeight="1" s="22">
-      <c r="B37" s="29" t="inlineStr">
-        <is>
-          <t>Absensa memvalidasi seluruh workbook sebelum menyimpan apa pun. Jika satu baris saja salah, seluruh impor ditolak: tidak ada siswa yang diubah dan tidak ada kelas yang diubah atau dibuat. Perbaiki semua kesalahan yang dilaporkan, lalu impor kembali.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1" s="22">
-      <c r="B40" s="53" t="inlineStr">
-        <is>
-          <t>Mengisi data siswa</t>
+      <c r="B36" s="53" t="n"/>
+    </row>
+    <row r="37" ht="25" customHeight="1" s="22">
+      <c r="B37" s="67" t="inlineStr">
+        <is>
+          <t>Jika impor gagal</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="n"/>
+      <c r="D37" s="28" t="n"/>
+      <c r="E37" s="28" t="n"/>
+      <c r="F37" s="28" t="n"/>
+      <c r="G37" s="28" t="n"/>
+      <c r="H37" s="26" t="n"/>
+    </row>
+    <row r="38" ht="57" customHeight="1" s="22">
+      <c r="B38" s="68" t="inlineStr">
+        <is>
+          <t>Absensa memeriksa seluruh data sebelum menyimpan perubahan. Impor berlaku semua-atau-tidak-sama-sekali: jika ada data atau file yang tidak valid, seluruh impor ditolak dan tidak ada siswa atau kelas yang disimpan sebagian. Baca laporan kesalahan, perbaiki file, lalu unggah kembali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="25" customHeight="1" s="22">
+      <c r="B40" s="67" t="inlineStr">
+        <is>
+          <t>Menggunakan data di luar Absensa</t>
         </is>
       </c>
       <c r="C40" s="28" t="n"/>
@@ -1311,68 +1382,56 @@
       <c r="G40" s="28" t="n"/>
       <c r="H40" s="26" t="n"/>
     </row>
-    <row r="41" ht="62" customHeight="1" s="22">
-      <c r="B41" s="29" t="inlineStr">
-        <is>
-          <t>Pertahankan ID siswa untuk pembaruan; kosongkan ID untuk siswa baru. NISN wajib tepat 10 digit dan disimpan sebagai teks agar nol di depan tidak hilang. STATUS: Aktif atau Tidak aktif. NOMOR WALI opsional, angka saja diawali 08 atau 628, maksimal 32 digit. Baris kosong diabaikan.</t>
+    <row r="41" ht="57" customHeight="1" s="22">
+      <c r="B41" s="68" t="inlineStr">
+        <is>
+          <t>Data hasil ekspor boleh digunakan untuk keperluan administrasi sekolah lainnya, seperti menyiapkan rapor atau mengolah data di sistem lain. Silakan salin dan olah data sesuai kebutuhan. Jika file akan diimpor kembali ke Absensa, pertahankan struktur, ID yang diperlukan, sel terlindungi, dan validasi yang tersedia.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="24" customHeight="1" s="22">
-      <c r="B44" s="53" t="inlineStr">
-        <is>
-          <t>Tanpa makro; finalisasi ID saat impor</t>
-        </is>
-      </c>
-      <c r="C44" s="28" t="n"/>
-      <c r="D44" s="28" t="n"/>
-      <c r="E44" s="28" t="n"/>
-      <c r="F44" s="28" t="n"/>
-      <c r="G44" s="28" t="n"/>
-      <c r="H44" s="26" t="n"/>
+      <c r="B44" s="53" t="n"/>
     </row>
     <row r="45" ht="100" customHeight="1" s="22">
-      <c r="B45" s="29" t="inlineStr">
-        <is>
-          <t>XLSX tanpa makro tidak dapat membuat ID otomatis saat pengisian lalu mengingatnya secara permanen. Karena itu ID N dialokasikan saat file dibuat dan difinalisasi oleh Absensa saat impor. Jika 100 baris habis, impor lalu unduh ulang untuk mendapat cadangan baru. Baris kelas tanpa ID tetap dapat diimpor, tetapi baru dapat dirujuk siswa setelah diekspor ulang. Jangan menimpa rumus siswa dengan nilai manual.</t>
-        </is>
-      </c>
+      <c r="B45" s="29" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="31">
     <mergeCell ref="B40:H40"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B5:H5"/>
     <mergeCell ref="B20:H20"/>
-    <mergeCell ref="B45:H45"/>
-    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="B32:H32"/>
     <mergeCell ref="D6:H6"/>
+    <mergeCell ref="B26:H26"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B35:H35"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B22:H22"/>
     <mergeCell ref="D7:H7"/>
-    <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B23:H23"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B14:H14"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="B38:H38"/>
     <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B34:H34"/>
     <mergeCell ref="B28:H28"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1395,8 +1454,8 @@
     <col width="15.89" customWidth="1" style="45" min="4" max="4"/>
     <col width="28.38" customWidth="1" style="45" min="5" max="5"/>
     <col width="15.89" customWidth="1" style="22" min="6" max="6"/>
-    <col width="34.06" customWidth="1" style="22" min="7" max="7"/>
-    <col width="15.89" customWidth="1" style="44" min="8" max="8"/>
+    <col width="15.89" customWidth="1" style="22" min="7" max="7"/>
+    <col width="34.06" customWidth="1" style="44" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1" s="22">
@@ -1425,1033 +1484,1034 @@
           <t>NOMOR WALI</t>
         </is>
       </c>
-      <c r="F1" s="48" t="inlineStr">
+      <c r="F1" s="47" t="inlineStr">
+        <is>
+          <t>ID KELAS</t>
+        </is>
+      </c>
+      <c r="G1" s="48" t="inlineStr">
         <is>
           <t>JENJANG</t>
         </is>
       </c>
-      <c r="G1" s="48" t="inlineStr">
+      <c r="H1" s="48" t="inlineStr">
         <is>
           <t>NAMA KELAS</t>
         </is>
       </c>
-      <c r="H1" s="47" t="inlineStr">
-        <is>
-          <t>ID KELAS</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="22">
-      <c r="A2" s="49" t="n"/>
-      <c r="B2" s="50" t="n"/>
-      <c r="C2" s="52" t="n"/>
-      <c r="D2" s="52" t="n"/>
-      <c r="E2" s="52" t="n"/>
-      <c r="F2" s="54" t="n"/>
-      <c r="G2" s="55" t="n"/>
-      <c r="H2" s="51" t="n"/>
+      <c r="A2" s="71" t="n"/>
+      <c r="B2" s="72" t="n"/>
+      <c r="C2" s="73" t="n"/>
+      <c r="D2" s="73" t="n"/>
+      <c r="E2" s="73" t="n"/>
+      <c r="F2" s="74" t="n"/>
+      <c r="G2" s="54" t="n"/>
+      <c r="H2" s="55" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="49" t="n"/>
-      <c r="B3" s="50" t="n"/>
-      <c r="C3" s="52" t="n"/>
-      <c r="D3" s="52" t="n"/>
-      <c r="E3" s="52" t="n"/>
-      <c r="F3" s="52" t="n"/>
+      <c r="A3" s="71" t="n"/>
+      <c r="B3" s="72" t="n"/>
+      <c r="C3" s="73" t="n"/>
+      <c r="D3" s="73" t="n"/>
+      <c r="E3" s="73" t="n"/>
+      <c r="F3" s="74" t="n"/>
       <c r="G3" s="52" t="n"/>
-      <c r="H3" s="51" t="n"/>
+      <c r="H3" s="52" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="49" t="n"/>
-      <c r="B4" s="50" t="n"/>
-      <c r="C4" s="52" t="n"/>
-      <c r="D4" s="52" t="n"/>
-      <c r="E4" s="52" t="n"/>
-      <c r="F4" s="52" t="n"/>
+      <c r="A4" s="71" t="n"/>
+      <c r="B4" s="72" t="n"/>
+      <c r="C4" s="73" t="n"/>
+      <c r="D4" s="73" t="n"/>
+      <c r="E4" s="73" t="n"/>
+      <c r="F4" s="74" t="n"/>
       <c r="G4" s="52" t="n"/>
-      <c r="H4" s="51" t="n"/>
+      <c r="H4" s="52" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="49" t="n"/>
-      <c r="B5" s="50" t="n"/>
-      <c r="C5" s="52" t="n"/>
-      <c r="D5" s="52" t="n"/>
-      <c r="E5" s="52" t="n"/>
-      <c r="F5" s="52" t="n"/>
+      <c r="A5" s="71" t="n"/>
+      <c r="B5" s="72" t="n"/>
+      <c r="C5" s="73" t="n"/>
+      <c r="D5" s="73" t="n"/>
+      <c r="E5" s="73" t="n"/>
+      <c r="F5" s="74" t="n"/>
       <c r="G5" s="52" t="n"/>
-      <c r="H5" s="51" t="n"/>
+      <c r="H5" s="52" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="49" t="n"/>
-      <c r="B6" s="50" t="n"/>
-      <c r="C6" s="52" t="n"/>
-      <c r="D6" s="52" t="n"/>
-      <c r="E6" s="52" t="n"/>
-      <c r="F6" s="52" t="n"/>
+      <c r="A6" s="71" t="n"/>
+      <c r="B6" s="72" t="n"/>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="73" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="74" t="n"/>
       <c r="G6" s="52" t="n"/>
-      <c r="H6" s="51" t="n"/>
+      <c r="H6" s="52" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="49" t="n"/>
-      <c r="B7" s="50" t="n"/>
-      <c r="C7" s="52" t="n"/>
-      <c r="D7" s="52" t="n"/>
-      <c r="E7" s="52" t="n"/>
-      <c r="F7" s="52" t="n"/>
+      <c r="A7" s="71" t="n"/>
+      <c r="B7" s="72" t="n"/>
+      <c r="C7" s="73" t="n"/>
+      <c r="D7" s="73" t="n"/>
+      <c r="E7" s="73" t="n"/>
+      <c r="F7" s="74" t="n"/>
       <c r="G7" s="52" t="n"/>
-      <c r="H7" s="51" t="n"/>
+      <c r="H7" s="52" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="49" t="n"/>
-      <c r="B8" s="50" t="n"/>
-      <c r="C8" s="52" t="n"/>
-      <c r="D8" s="52" t="n"/>
-      <c r="E8" s="52" t="n"/>
-      <c r="F8" s="52" t="n"/>
+      <c r="A8" s="71" t="n"/>
+      <c r="B8" s="72" t="n"/>
+      <c r="C8" s="73" t="n"/>
+      <c r="D8" s="73" t="n"/>
+      <c r="E8" s="73" t="n"/>
+      <c r="F8" s="74" t="n"/>
       <c r="G8" s="52" t="n"/>
-      <c r="H8" s="51" t="n"/>
+      <c r="H8" s="52" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="49" t="n"/>
-      <c r="B9" s="50" t="n"/>
-      <c r="C9" s="52" t="n"/>
-      <c r="D9" s="52" t="n"/>
-      <c r="E9" s="52" t="n"/>
-      <c r="F9" s="52" t="n"/>
+      <c r="A9" s="71" t="n"/>
+      <c r="B9" s="72" t="n"/>
+      <c r="C9" s="73" t="n"/>
+      <c r="D9" s="73" t="n"/>
+      <c r="E9" s="73" t="n"/>
+      <c r="F9" s="74" t="n"/>
       <c r="G9" s="52" t="n"/>
-      <c r="H9" s="51" t="n"/>
+      <c r="H9" s="52" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="49" t="n"/>
-      <c r="B10" s="50" t="n"/>
-      <c r="C10" s="52" t="n"/>
-      <c r="D10" s="52" t="n"/>
-      <c r="E10" s="52" t="n"/>
-      <c r="F10" s="52" t="n"/>
+      <c r="A10" s="71" t="n"/>
+      <c r="B10" s="72" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="74" t="n"/>
       <c r="G10" s="52" t="n"/>
-      <c r="H10" s="51" t="n"/>
+      <c r="H10" s="52" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="49" t="n"/>
-      <c r="B11" s="50" t="n"/>
-      <c r="C11" s="52" t="n"/>
-      <c r="D11" s="52" t="n"/>
-      <c r="E11" s="52" t="n"/>
-      <c r="F11" s="52" t="n"/>
+      <c r="A11" s="71" t="n"/>
+      <c r="B11" s="72" t="n"/>
+      <c r="C11" s="73" t="n"/>
+      <c r="D11" s="73" t="n"/>
+      <c r="E11" s="73" t="n"/>
+      <c r="F11" s="74" t="n"/>
       <c r="G11" s="52" t="n"/>
-      <c r="H11" s="51" t="n"/>
+      <c r="H11" s="52" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="49" t="n"/>
-      <c r="B12" s="50" t="n"/>
-      <c r="C12" s="52" t="n"/>
-      <c r="D12" s="52" t="n"/>
-      <c r="E12" s="52" t="n"/>
-      <c r="F12" s="52" t="n"/>
+      <c r="A12" s="71" t="n"/>
+      <c r="B12" s="72" t="n"/>
+      <c r="C12" s="73" t="n"/>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="73" t="n"/>
+      <c r="F12" s="74" t="n"/>
       <c r="G12" s="52" t="n"/>
-      <c r="H12" s="51" t="n"/>
+      <c r="H12" s="52" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="49" t="n"/>
-      <c r="B13" s="50" t="n"/>
-      <c r="C13" s="52" t="n"/>
-      <c r="D13" s="52" t="n"/>
-      <c r="E13" s="52" t="n"/>
-      <c r="F13" s="52" t="n"/>
+      <c r="A13" s="71" t="n"/>
+      <c r="B13" s="72" t="n"/>
+      <c r="C13" s="73" t="n"/>
+      <c r="D13" s="73" t="n"/>
+      <c r="E13" s="73" t="n"/>
+      <c r="F13" s="74" t="n"/>
       <c r="G13" s="52" t="n"/>
-      <c r="H13" s="51" t="n"/>
+      <c r="H13" s="52" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="49" t="n"/>
-      <c r="B14" s="50" t="n"/>
-      <c r="C14" s="52" t="n"/>
-      <c r="D14" s="52" t="n"/>
-      <c r="E14" s="52" t="n"/>
-      <c r="F14" s="52" t="n"/>
+      <c r="A14" s="71" t="n"/>
+      <c r="B14" s="72" t="n"/>
+      <c r="C14" s="73" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="73" t="n"/>
+      <c r="F14" s="74" t="n"/>
       <c r="G14" s="52" t="n"/>
-      <c r="H14" s="51" t="n"/>
+      <c r="H14" s="52" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="49" t="n"/>
-      <c r="B15" s="50" t="n"/>
-      <c r="C15" s="52" t="n"/>
-      <c r="D15" s="52" t="n"/>
-      <c r="E15" s="52" t="n"/>
-      <c r="F15" s="52" t="n"/>
+      <c r="A15" s="71" t="n"/>
+      <c r="B15" s="72" t="n"/>
+      <c r="C15" s="73" t="n"/>
+      <c r="D15" s="73" t="n"/>
+      <c r="E15" s="73" t="n"/>
+      <c r="F15" s="74" t="n"/>
       <c r="G15" s="52" t="n"/>
-      <c r="H15" s="51" t="n"/>
+      <c r="H15" s="52" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="49" t="n"/>
-      <c r="B16" s="50" t="n"/>
-      <c r="C16" s="52" t="n"/>
-      <c r="D16" s="52" t="n"/>
-      <c r="E16" s="52" t="n"/>
-      <c r="F16" s="52" t="n"/>
+      <c r="A16" s="71" t="n"/>
+      <c r="B16" s="72" t="n"/>
+      <c r="C16" s="73" t="n"/>
+      <c r="D16" s="73" t="n"/>
+      <c r="E16" s="73" t="n"/>
+      <c r="F16" s="74" t="n"/>
       <c r="G16" s="52" t="n"/>
-      <c r="H16" s="51" t="n"/>
+      <c r="H16" s="52" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="49" t="n"/>
-      <c r="B17" s="50" t="n"/>
-      <c r="C17" s="52" t="n"/>
-      <c r="D17" s="52" t="n"/>
-      <c r="E17" s="52" t="n"/>
-      <c r="F17" s="52" t="n"/>
+      <c r="A17" s="71" t="n"/>
+      <c r="B17" s="72" t="n"/>
+      <c r="C17" s="73" t="n"/>
+      <c r="D17" s="73" t="n"/>
+      <c r="E17" s="73" t="n"/>
+      <c r="F17" s="74" t="n"/>
       <c r="G17" s="52" t="n"/>
-      <c r="H17" s="51" t="n"/>
+      <c r="H17" s="52" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="49" t="n"/>
-      <c r="B18" s="50" t="n"/>
-      <c r="C18" s="52" t="n"/>
-      <c r="D18" s="52" t="n"/>
-      <c r="E18" s="52" t="n"/>
-      <c r="F18" s="52" t="n"/>
+      <c r="A18" s="71" t="n"/>
+      <c r="B18" s="72" t="n"/>
+      <c r="C18" s="73" t="n"/>
+      <c r="D18" s="73" t="n"/>
+      <c r="E18" s="73" t="n"/>
+      <c r="F18" s="74" t="n"/>
       <c r="G18" s="52" t="n"/>
-      <c r="H18" s="51" t="n"/>
+      <c r="H18" s="52" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="49" t="n"/>
-      <c r="B19" s="50" t="n"/>
-      <c r="C19" s="52" t="n"/>
-      <c r="D19" s="52" t="n"/>
-      <c r="E19" s="52" t="n"/>
-      <c r="F19" s="52" t="n"/>
+      <c r="A19" s="71" t="n"/>
+      <c r="B19" s="72" t="n"/>
+      <c r="C19" s="73" t="n"/>
+      <c r="D19" s="73" t="n"/>
+      <c r="E19" s="73" t="n"/>
+      <c r="F19" s="74" t="n"/>
       <c r="G19" s="52" t="n"/>
-      <c r="H19" s="51" t="n"/>
+      <c r="H19" s="52" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="49" t="n"/>
-      <c r="B20" s="50" t="n"/>
-      <c r="C20" s="52" t="n"/>
-      <c r="D20" s="52" t="n"/>
-      <c r="E20" s="52" t="n"/>
-      <c r="F20" s="52" t="n"/>
+      <c r="A20" s="71" t="n"/>
+      <c r="B20" s="72" t="n"/>
+      <c r="C20" s="73" t="n"/>
+      <c r="D20" s="73" t="n"/>
+      <c r="E20" s="73" t="n"/>
+      <c r="F20" s="74" t="n"/>
       <c r="G20" s="52" t="n"/>
-      <c r="H20" s="51" t="n"/>
+      <c r="H20" s="52" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="49" t="n"/>
-      <c r="B21" s="50" t="n"/>
-      <c r="C21" s="52" t="n"/>
-      <c r="D21" s="52" t="n"/>
-      <c r="E21" s="52" t="n"/>
-      <c r="F21" s="52" t="n"/>
+      <c r="A21" s="71" t="n"/>
+      <c r="B21" s="72" t="n"/>
+      <c r="C21" s="73" t="n"/>
+      <c r="D21" s="73" t="n"/>
+      <c r="E21" s="73" t="n"/>
+      <c r="F21" s="74" t="n"/>
       <c r="G21" s="52" t="n"/>
-      <c r="H21" s="51" t="n"/>
+      <c r="H21" s="52" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="49" t="n"/>
-      <c r="B22" s="50" t="n"/>
-      <c r="C22" s="52" t="n"/>
-      <c r="D22" s="52" t="n"/>
-      <c r="E22" s="52" t="n"/>
-      <c r="F22" s="52" t="n"/>
+      <c r="A22" s="71" t="n"/>
+      <c r="B22" s="72" t="n"/>
+      <c r="C22" s="73" t="n"/>
+      <c r="D22" s="73" t="n"/>
+      <c r="E22" s="73" t="n"/>
+      <c r="F22" s="74" t="n"/>
       <c r="G22" s="52" t="n"/>
-      <c r="H22" s="51" t="n"/>
+      <c r="H22" s="52" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="49" t="n"/>
-      <c r="B23" s="50" t="n"/>
-      <c r="C23" s="52" t="n"/>
-      <c r="D23" s="52" t="n"/>
-      <c r="E23" s="52" t="n"/>
-      <c r="F23" s="52" t="n"/>
+      <c r="A23" s="71" t="n"/>
+      <c r="B23" s="72" t="n"/>
+      <c r="C23" s="73" t="n"/>
+      <c r="D23" s="73" t="n"/>
+      <c r="E23" s="73" t="n"/>
+      <c r="F23" s="74" t="n"/>
       <c r="G23" s="52" t="n"/>
-      <c r="H23" s="51" t="n"/>
+      <c r="H23" s="52" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="49" t="n"/>
-      <c r="B24" s="50" t="n"/>
-      <c r="C24" s="52" t="n"/>
-      <c r="D24" s="52" t="n"/>
-      <c r="E24" s="52" t="n"/>
-      <c r="F24" s="52" t="n"/>
+      <c r="A24" s="71" t="n"/>
+      <c r="B24" s="72" t="n"/>
+      <c r="C24" s="73" t="n"/>
+      <c r="D24" s="73" t="n"/>
+      <c r="E24" s="73" t="n"/>
+      <c r="F24" s="74" t="n"/>
       <c r="G24" s="52" t="n"/>
-      <c r="H24" s="51" t="n"/>
+      <c r="H24" s="52" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="49" t="n"/>
-      <c r="B25" s="50" t="n"/>
-      <c r="C25" s="52" t="n"/>
-      <c r="D25" s="52" t="n"/>
-      <c r="E25" s="52" t="n"/>
-      <c r="F25" s="52" t="n"/>
+      <c r="A25" s="71" t="n"/>
+      <c r="B25" s="72" t="n"/>
+      <c r="C25" s="73" t="n"/>
+      <c r="D25" s="73" t="n"/>
+      <c r="E25" s="73" t="n"/>
+      <c r="F25" s="74" t="n"/>
       <c r="G25" s="52" t="n"/>
-      <c r="H25" s="51" t="n"/>
+      <c r="H25" s="52" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="49" t="n"/>
-      <c r="B26" s="50" t="n"/>
-      <c r="C26" s="52" t="n"/>
-      <c r="D26" s="52" t="n"/>
-      <c r="E26" s="52" t="n"/>
-      <c r="F26" s="52" t="n"/>
+      <c r="A26" s="71" t="n"/>
+      <c r="B26" s="72" t="n"/>
+      <c r="C26" s="73" t="n"/>
+      <c r="D26" s="73" t="n"/>
+      <c r="E26" s="73" t="n"/>
+      <c r="F26" s="74" t="n"/>
       <c r="G26" s="52" t="n"/>
-      <c r="H26" s="51" t="n"/>
+      <c r="H26" s="52" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="49" t="n"/>
-      <c r="B27" s="50" t="n"/>
-      <c r="C27" s="52" t="n"/>
-      <c r="D27" s="52" t="n"/>
-      <c r="E27" s="52" t="n"/>
-      <c r="F27" s="52" t="n"/>
+      <c r="A27" s="71" t="n"/>
+      <c r="B27" s="72" t="n"/>
+      <c r="C27" s="73" t="n"/>
+      <c r="D27" s="73" t="n"/>
+      <c r="E27" s="73" t="n"/>
+      <c r="F27" s="74" t="n"/>
       <c r="G27" s="52" t="n"/>
-      <c r="H27" s="51" t="n"/>
+      <c r="H27" s="52" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="49" t="n"/>
-      <c r="B28" s="50" t="n"/>
-      <c r="C28" s="52" t="n"/>
-      <c r="D28" s="52" t="n"/>
-      <c r="E28" s="52" t="n"/>
-      <c r="F28" s="52" t="n"/>
+      <c r="A28" s="71" t="n"/>
+      <c r="B28" s="72" t="n"/>
+      <c r="C28" s="73" t="n"/>
+      <c r="D28" s="73" t="n"/>
+      <c r="E28" s="73" t="n"/>
+      <c r="F28" s="74" t="n"/>
       <c r="G28" s="52" t="n"/>
-      <c r="H28" s="51" t="n"/>
+      <c r="H28" s="52" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="49" t="n"/>
-      <c r="B29" s="50" t="n"/>
-      <c r="C29" s="52" t="n"/>
-      <c r="D29" s="52" t="n"/>
-      <c r="E29" s="52" t="n"/>
-      <c r="F29" s="52" t="n"/>
+      <c r="A29" s="71" t="n"/>
+      <c r="B29" s="72" t="n"/>
+      <c r="C29" s="73" t="n"/>
+      <c r="D29" s="73" t="n"/>
+      <c r="E29" s="73" t="n"/>
+      <c r="F29" s="74" t="n"/>
       <c r="G29" s="52" t="n"/>
-      <c r="H29" s="51" t="n"/>
+      <c r="H29" s="52" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="49" t="n"/>
-      <c r="B30" s="50" t="n"/>
-      <c r="C30" s="52" t="n"/>
-      <c r="D30" s="52" t="n"/>
-      <c r="E30" s="52" t="n"/>
-      <c r="F30" s="52" t="n"/>
+      <c r="A30" s="71" t="n"/>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="73" t="n"/>
+      <c r="D30" s="73" t="n"/>
+      <c r="E30" s="73" t="n"/>
+      <c r="F30" s="74" t="n"/>
       <c r="G30" s="52" t="n"/>
-      <c r="H30" s="51" t="n"/>
+      <c r="H30" s="52" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="49" t="n"/>
-      <c r="B31" s="50" t="n"/>
-      <c r="C31" s="52" t="n"/>
-      <c r="D31" s="52" t="n"/>
-      <c r="E31" s="52" t="n"/>
-      <c r="F31" s="52" t="n"/>
+      <c r="A31" s="71" t="n"/>
+      <c r="B31" s="72" t="n"/>
+      <c r="C31" s="73" t="n"/>
+      <c r="D31" s="73" t="n"/>
+      <c r="E31" s="73" t="n"/>
+      <c r="F31" s="74" t="n"/>
       <c r="G31" s="52" t="n"/>
-      <c r="H31" s="51" t="n"/>
+      <c r="H31" s="52" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="n"/>
-      <c r="B32" s="50" t="n"/>
-      <c r="C32" s="52" t="n"/>
-      <c r="D32" s="52" t="n"/>
-      <c r="E32" s="52" t="n"/>
-      <c r="F32" s="52" t="n"/>
+      <c r="A32" s="71" t="n"/>
+      <c r="B32" s="72" t="n"/>
+      <c r="C32" s="73" t="n"/>
+      <c r="D32" s="73" t="n"/>
+      <c r="E32" s="73" t="n"/>
+      <c r="F32" s="74" t="n"/>
       <c r="G32" s="52" t="n"/>
-      <c r="H32" s="51" t="n"/>
+      <c r="H32" s="52" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="49" t="n"/>
-      <c r="B33" s="50" t="n"/>
-      <c r="C33" s="52" t="n"/>
-      <c r="D33" s="52" t="n"/>
-      <c r="E33" s="52" t="n"/>
-      <c r="F33" s="52" t="n"/>
+      <c r="A33" s="71" t="n"/>
+      <c r="B33" s="72" t="n"/>
+      <c r="C33" s="73" t="n"/>
+      <c r="D33" s="73" t="n"/>
+      <c r="E33" s="73" t="n"/>
+      <c r="F33" s="74" t="n"/>
       <c r="G33" s="52" t="n"/>
-      <c r="H33" s="51" t="n"/>
+      <c r="H33" s="52" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="49" t="n"/>
-      <c r="B34" s="50" t="n"/>
-      <c r="C34" s="52" t="n"/>
-      <c r="D34" s="52" t="n"/>
-      <c r="E34" s="52" t="n"/>
-      <c r="F34" s="52" t="n"/>
+      <c r="A34" s="71" t="n"/>
+      <c r="B34" s="72" t="n"/>
+      <c r="C34" s="73" t="n"/>
+      <c r="D34" s="73" t="n"/>
+      <c r="E34" s="73" t="n"/>
+      <c r="F34" s="74" t="n"/>
       <c r="G34" s="52" t="n"/>
-      <c r="H34" s="51" t="n"/>
+      <c r="H34" s="52" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="49" t="n"/>
-      <c r="B35" s="50" t="n"/>
-      <c r="C35" s="52" t="n"/>
-      <c r="D35" s="52" t="n"/>
-      <c r="E35" s="52" t="n"/>
-      <c r="F35" s="52" t="n"/>
+      <c r="A35" s="71" t="n"/>
+      <c r="B35" s="72" t="n"/>
+      <c r="C35" s="73" t="n"/>
+      <c r="D35" s="73" t="n"/>
+      <c r="E35" s="73" t="n"/>
+      <c r="F35" s="74" t="n"/>
       <c r="G35" s="52" t="n"/>
-      <c r="H35" s="51" t="n"/>
+      <c r="H35" s="52" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="49" t="n"/>
-      <c r="B36" s="50" t="n"/>
-      <c r="C36" s="52" t="n"/>
-      <c r="D36" s="52" t="n"/>
-      <c r="E36" s="52" t="n"/>
-      <c r="F36" s="52" t="n"/>
+      <c r="A36" s="71" t="n"/>
+      <c r="B36" s="72" t="n"/>
+      <c r="C36" s="73" t="n"/>
+      <c r="D36" s="73" t="n"/>
+      <c r="E36" s="73" t="n"/>
+      <c r="F36" s="74" t="n"/>
       <c r="G36" s="52" t="n"/>
-      <c r="H36" s="51" t="n"/>
+      <c r="H36" s="52" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="49" t="n"/>
-      <c r="B37" s="50" t="n"/>
-      <c r="C37" s="52" t="n"/>
-      <c r="D37" s="52" t="n"/>
-      <c r="E37" s="52" t="n"/>
-      <c r="F37" s="52" t="n"/>
+      <c r="A37" s="71" t="n"/>
+      <c r="B37" s="72" t="n"/>
+      <c r="C37" s="73" t="n"/>
+      <c r="D37" s="73" t="n"/>
+      <c r="E37" s="73" t="n"/>
+      <c r="F37" s="74" t="n"/>
       <c r="G37" s="52" t="n"/>
-      <c r="H37" s="51" t="n"/>
+      <c r="H37" s="52" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="49" t="n"/>
-      <c r="B38" s="50" t="n"/>
-      <c r="C38" s="52" t="n"/>
-      <c r="D38" s="52" t="n"/>
-      <c r="E38" s="52" t="n"/>
-      <c r="F38" s="52" t="n"/>
+      <c r="A38" s="71" t="n"/>
+      <c r="B38" s="72" t="n"/>
+      <c r="C38" s="73" t="n"/>
+      <c r="D38" s="73" t="n"/>
+      <c r="E38" s="73" t="n"/>
+      <c r="F38" s="74" t="n"/>
       <c r="G38" s="52" t="n"/>
-      <c r="H38" s="51" t="n"/>
+      <c r="H38" s="52" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="49" t="n"/>
-      <c r="B39" s="50" t="n"/>
-      <c r="C39" s="52" t="n"/>
-      <c r="D39" s="52" t="n"/>
-      <c r="E39" s="52" t="n"/>
-      <c r="F39" s="52" t="n"/>
+      <c r="A39" s="71" t="n"/>
+      <c r="B39" s="72" t="n"/>
+      <c r="C39" s="73" t="n"/>
+      <c r="D39" s="73" t="n"/>
+      <c r="E39" s="73" t="n"/>
+      <c r="F39" s="74" t="n"/>
       <c r="G39" s="52" t="n"/>
-      <c r="H39" s="51" t="n"/>
+      <c r="H39" s="52" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="49" t="n"/>
-      <c r="B40" s="50" t="n"/>
-      <c r="C40" s="52" t="n"/>
-      <c r="D40" s="52" t="n"/>
-      <c r="E40" s="52" t="n"/>
-      <c r="F40" s="52" t="n"/>
+      <c r="A40" s="71" t="n"/>
+      <c r="B40" s="72" t="n"/>
+      <c r="C40" s="73" t="n"/>
+      <c r="D40" s="73" t="n"/>
+      <c r="E40" s="73" t="n"/>
+      <c r="F40" s="74" t="n"/>
       <c r="G40" s="52" t="n"/>
-      <c r="H40" s="51" t="n"/>
+      <c r="H40" s="52" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="49" t="n"/>
-      <c r="B41" s="50" t="n"/>
-      <c r="C41" s="52" t="n"/>
-      <c r="D41" s="52" t="n"/>
-      <c r="E41" s="52" t="n"/>
-      <c r="F41" s="52" t="n"/>
+      <c r="A41" s="71" t="n"/>
+      <c r="B41" s="72" t="n"/>
+      <c r="C41" s="73" t="n"/>
+      <c r="D41" s="73" t="n"/>
+      <c r="E41" s="73" t="n"/>
+      <c r="F41" s="74" t="n"/>
       <c r="G41" s="52" t="n"/>
-      <c r="H41" s="51" t="n"/>
+      <c r="H41" s="52" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="49" t="n"/>
-      <c r="B42" s="50" t="n"/>
-      <c r="C42" s="52" t="n"/>
-      <c r="D42" s="52" t="n"/>
-      <c r="E42" s="52" t="n"/>
-      <c r="F42" s="52" t="n"/>
+      <c r="A42" s="71" t="n"/>
+      <c r="B42" s="72" t="n"/>
+      <c r="C42" s="73" t="n"/>
+      <c r="D42" s="73" t="n"/>
+      <c r="E42" s="73" t="n"/>
+      <c r="F42" s="74" t="n"/>
       <c r="G42" s="52" t="n"/>
-      <c r="H42" s="51" t="n"/>
+      <c r="H42" s="52" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="49" t="n"/>
-      <c r="B43" s="50" t="n"/>
-      <c r="C43" s="52" t="n"/>
-      <c r="D43" s="52" t="n"/>
-      <c r="E43" s="52" t="n"/>
-      <c r="F43" s="52" t="n"/>
+      <c r="A43" s="71" t="n"/>
+      <c r="B43" s="72" t="n"/>
+      <c r="C43" s="73" t="n"/>
+      <c r="D43" s="73" t="n"/>
+      <c r="E43" s="73" t="n"/>
+      <c r="F43" s="74" t="n"/>
       <c r="G43" s="52" t="n"/>
-      <c r="H43" s="51" t="n"/>
+      <c r="H43" s="52" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="49" t="n"/>
-      <c r="B44" s="50" t="n"/>
-      <c r="C44" s="52" t="n"/>
-      <c r="D44" s="52" t="n"/>
-      <c r="E44" s="52" t="n"/>
-      <c r="F44" s="52" t="n"/>
+      <c r="A44" s="71" t="n"/>
+      <c r="B44" s="72" t="n"/>
+      <c r="C44" s="73" t="n"/>
+      <c r="D44" s="73" t="n"/>
+      <c r="E44" s="73" t="n"/>
+      <c r="F44" s="74" t="n"/>
       <c r="G44" s="52" t="n"/>
-      <c r="H44" s="51" t="n"/>
+      <c r="H44" s="52" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="49" t="n"/>
-      <c r="B45" s="50" t="n"/>
-      <c r="C45" s="52" t="n"/>
-      <c r="D45" s="52" t="n"/>
-      <c r="E45" s="52" t="n"/>
-      <c r="F45" s="52" t="n"/>
+      <c r="A45" s="71" t="n"/>
+      <c r="B45" s="72" t="n"/>
+      <c r="C45" s="73" t="n"/>
+      <c r="D45" s="73" t="n"/>
+      <c r="E45" s="73" t="n"/>
+      <c r="F45" s="74" t="n"/>
       <c r="G45" s="52" t="n"/>
-      <c r="H45" s="51" t="n"/>
+      <c r="H45" s="52" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="49" t="n"/>
-      <c r="B46" s="50" t="n"/>
-      <c r="C46" s="52" t="n"/>
-      <c r="D46" s="52" t="n"/>
-      <c r="E46" s="52" t="n"/>
-      <c r="F46" s="52" t="n"/>
+      <c r="A46" s="71" t="n"/>
+      <c r="B46" s="72" t="n"/>
+      <c r="C46" s="73" t="n"/>
+      <c r="D46" s="73" t="n"/>
+      <c r="E46" s="73" t="n"/>
+      <c r="F46" s="74" t="n"/>
       <c r="G46" s="52" t="n"/>
-      <c r="H46" s="51" t="n"/>
+      <c r="H46" s="52" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="49" t="n"/>
-      <c r="B47" s="50" t="n"/>
-      <c r="C47" s="52" t="n"/>
-      <c r="D47" s="52" t="n"/>
-      <c r="E47" s="52" t="n"/>
-      <c r="F47" s="52" t="n"/>
+      <c r="A47" s="71" t="n"/>
+      <c r="B47" s="72" t="n"/>
+      <c r="C47" s="73" t="n"/>
+      <c r="D47" s="73" t="n"/>
+      <c r="E47" s="73" t="n"/>
+      <c r="F47" s="74" t="n"/>
       <c r="G47" s="52" t="n"/>
-      <c r="H47" s="51" t="n"/>
+      <c r="H47" s="52" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="49" t="n"/>
-      <c r="B48" s="50" t="n"/>
-      <c r="C48" s="52" t="n"/>
-      <c r="D48" s="52" t="n"/>
-      <c r="E48" s="52" t="n"/>
-      <c r="F48" s="52" t="n"/>
+      <c r="A48" s="71" t="n"/>
+      <c r="B48" s="72" t="n"/>
+      <c r="C48" s="73" t="n"/>
+      <c r="D48" s="73" t="n"/>
+      <c r="E48" s="73" t="n"/>
+      <c r="F48" s="74" t="n"/>
       <c r="G48" s="52" t="n"/>
-      <c r="H48" s="51" t="n"/>
+      <c r="H48" s="52" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="49" t="n"/>
-      <c r="B49" s="50" t="n"/>
-      <c r="C49" s="52" t="n"/>
-      <c r="D49" s="52" t="n"/>
-      <c r="E49" s="52" t="n"/>
-      <c r="F49" s="52" t="n"/>
+      <c r="A49" s="71" t="n"/>
+      <c r="B49" s="72" t="n"/>
+      <c r="C49" s="73" t="n"/>
+      <c r="D49" s="73" t="n"/>
+      <c r="E49" s="73" t="n"/>
+      <c r="F49" s="74" t="n"/>
       <c r="G49" s="52" t="n"/>
-      <c r="H49" s="51" t="n"/>
+      <c r="H49" s="52" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="49" t="n"/>
-      <c r="B50" s="50" t="n"/>
-      <c r="C50" s="52" t="n"/>
-      <c r="D50" s="52" t="n"/>
-      <c r="E50" s="52" t="n"/>
-      <c r="F50" s="52" t="n"/>
+      <c r="A50" s="71" t="n"/>
+      <c r="B50" s="72" t="n"/>
+      <c r="C50" s="73" t="n"/>
+      <c r="D50" s="73" t="n"/>
+      <c r="E50" s="73" t="n"/>
+      <c r="F50" s="74" t="n"/>
       <c r="G50" s="52" t="n"/>
-      <c r="H50" s="51" t="n"/>
+      <c r="H50" s="52" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="49" t="n"/>
-      <c r="B51" s="50" t="n"/>
-      <c r="C51" s="52" t="n"/>
-      <c r="D51" s="52" t="n"/>
-      <c r="E51" s="52" t="n"/>
-      <c r="F51" s="52" t="n"/>
+      <c r="A51" s="71" t="n"/>
+      <c r="B51" s="72" t="n"/>
+      <c r="C51" s="73" t="n"/>
+      <c r="D51" s="73" t="n"/>
+      <c r="E51" s="73" t="n"/>
+      <c r="F51" s="74" t="n"/>
       <c r="G51" s="52" t="n"/>
-      <c r="H51" s="51" t="n"/>
+      <c r="H51" s="52" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="49" t="n"/>
-      <c r="B52" s="50" t="n"/>
-      <c r="C52" s="52" t="n"/>
-      <c r="D52" s="52" t="n"/>
-      <c r="E52" s="52" t="n"/>
-      <c r="F52" s="52" t="n"/>
+      <c r="A52" s="71" t="n"/>
+      <c r="B52" s="72" t="n"/>
+      <c r="C52" s="73" t="n"/>
+      <c r="D52" s="73" t="n"/>
+      <c r="E52" s="73" t="n"/>
+      <c r="F52" s="74" t="n"/>
       <c r="G52" s="52" t="n"/>
-      <c r="H52" s="51" t="n"/>
+      <c r="H52" s="52" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="49" t="n"/>
-      <c r="B53" s="50" t="n"/>
-      <c r="C53" s="52" t="n"/>
-      <c r="D53" s="52" t="n"/>
-      <c r="E53" s="52" t="n"/>
-      <c r="F53" s="52" t="n"/>
+      <c r="A53" s="71" t="n"/>
+      <c r="B53" s="72" t="n"/>
+      <c r="C53" s="73" t="n"/>
+      <c r="D53" s="73" t="n"/>
+      <c r="E53" s="73" t="n"/>
+      <c r="F53" s="74" t="n"/>
       <c r="G53" s="52" t="n"/>
-      <c r="H53" s="51" t="n"/>
+      <c r="H53" s="52" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="49" t="n"/>
-      <c r="B54" s="50" t="n"/>
-      <c r="C54" s="52" t="n"/>
-      <c r="D54" s="52" t="n"/>
-      <c r="E54" s="52" t="n"/>
-      <c r="F54" s="52" t="n"/>
+      <c r="A54" s="71" t="n"/>
+      <c r="B54" s="72" t="n"/>
+      <c r="C54" s="73" t="n"/>
+      <c r="D54" s="73" t="n"/>
+      <c r="E54" s="73" t="n"/>
+      <c r="F54" s="74" t="n"/>
       <c r="G54" s="52" t="n"/>
-      <c r="H54" s="51" t="n"/>
+      <c r="H54" s="52" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="49" t="n"/>
-      <c r="B55" s="50" t="n"/>
-      <c r="C55" s="52" t="n"/>
-      <c r="D55" s="52" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="52" t="n"/>
+      <c r="A55" s="71" t="n"/>
+      <c r="B55" s="72" t="n"/>
+      <c r="C55" s="73" t="n"/>
+      <c r="D55" s="73" t="n"/>
+      <c r="E55" s="73" t="n"/>
+      <c r="F55" s="74" t="n"/>
       <c r="G55" s="52" t="n"/>
-      <c r="H55" s="51" t="n"/>
+      <c r="H55" s="52" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="49" t="n"/>
-      <c r="B56" s="50" t="n"/>
-      <c r="C56" s="52" t="n"/>
-      <c r="D56" s="52" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="52" t="n"/>
+      <c r="A56" s="71" t="n"/>
+      <c r="B56" s="72" t="n"/>
+      <c r="C56" s="73" t="n"/>
+      <c r="D56" s="73" t="n"/>
+      <c r="E56" s="73" t="n"/>
+      <c r="F56" s="74" t="n"/>
       <c r="G56" s="52" t="n"/>
-      <c r="H56" s="51" t="n"/>
+      <c r="H56" s="52" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="49" t="n"/>
-      <c r="B57" s="50" t="n"/>
-      <c r="C57" s="52" t="n"/>
-      <c r="D57" s="52" t="n"/>
-      <c r="E57" s="52" t="n"/>
-      <c r="F57" s="52" t="n"/>
+      <c r="A57" s="71" t="n"/>
+      <c r="B57" s="72" t="n"/>
+      <c r="C57" s="73" t="n"/>
+      <c r="D57" s="73" t="n"/>
+      <c r="E57" s="73" t="n"/>
+      <c r="F57" s="74" t="n"/>
       <c r="G57" s="52" t="n"/>
-      <c r="H57" s="51" t="n"/>
+      <c r="H57" s="52" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="49" t="n"/>
-      <c r="B58" s="50" t="n"/>
-      <c r="C58" s="52" t="n"/>
-      <c r="D58" s="52" t="n"/>
-      <c r="E58" s="52" t="n"/>
-      <c r="F58" s="52" t="n"/>
+      <c r="A58" s="71" t="n"/>
+      <c r="B58" s="72" t="n"/>
+      <c r="C58" s="73" t="n"/>
+      <c r="D58" s="73" t="n"/>
+      <c r="E58" s="73" t="n"/>
+      <c r="F58" s="74" t="n"/>
       <c r="G58" s="52" t="n"/>
-      <c r="H58" s="51" t="n"/>
+      <c r="H58" s="52" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="49" t="n"/>
-      <c r="B59" s="50" t="n"/>
-      <c r="C59" s="52" t="n"/>
-      <c r="D59" s="52" t="n"/>
-      <c r="E59" s="52" t="n"/>
-      <c r="F59" s="52" t="n"/>
+      <c r="A59" s="71" t="n"/>
+      <c r="B59" s="72" t="n"/>
+      <c r="C59" s="73" t="n"/>
+      <c r="D59" s="73" t="n"/>
+      <c r="E59" s="73" t="n"/>
+      <c r="F59" s="74" t="n"/>
       <c r="G59" s="52" t="n"/>
-      <c r="H59" s="51" t="n"/>
+      <c r="H59" s="52" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="49" t="n"/>
-      <c r="B60" s="50" t="n"/>
-      <c r="C60" s="52" t="n"/>
-      <c r="D60" s="52" t="n"/>
-      <c r="E60" s="52" t="n"/>
-      <c r="F60" s="52" t="n"/>
+      <c r="A60" s="71" t="n"/>
+      <c r="B60" s="72" t="n"/>
+      <c r="C60" s="73" t="n"/>
+      <c r="D60" s="73" t="n"/>
+      <c r="E60" s="73" t="n"/>
+      <c r="F60" s="74" t="n"/>
       <c r="G60" s="52" t="n"/>
-      <c r="H60" s="51" t="n"/>
+      <c r="H60" s="52" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="49" t="n"/>
-      <c r="B61" s="50" t="n"/>
-      <c r="C61" s="52" t="n"/>
-      <c r="D61" s="52" t="n"/>
-      <c r="E61" s="52" t="n"/>
-      <c r="F61" s="52" t="n"/>
+      <c r="A61" s="71" t="n"/>
+      <c r="B61" s="72" t="n"/>
+      <c r="C61" s="73" t="n"/>
+      <c r="D61" s="73" t="n"/>
+      <c r="E61" s="73" t="n"/>
+      <c r="F61" s="74" t="n"/>
       <c r="G61" s="52" t="n"/>
-      <c r="H61" s="51" t="n"/>
+      <c r="H61" s="52" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="49" t="n"/>
-      <c r="B62" s="50" t="n"/>
-      <c r="C62" s="52" t="n"/>
-      <c r="D62" s="52" t="n"/>
-      <c r="E62" s="52" t="n"/>
-      <c r="F62" s="52" t="n"/>
+      <c r="A62" s="71" t="n"/>
+      <c r="B62" s="72" t="n"/>
+      <c r="C62" s="73" t="n"/>
+      <c r="D62" s="73" t="n"/>
+      <c r="E62" s="73" t="n"/>
+      <c r="F62" s="74" t="n"/>
       <c r="G62" s="52" t="n"/>
-      <c r="H62" s="51" t="n"/>
+      <c r="H62" s="52" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="49" t="n"/>
-      <c r="B63" s="50" t="n"/>
-      <c r="C63" s="52" t="n"/>
-      <c r="D63" s="52" t="n"/>
-      <c r="E63" s="52" t="n"/>
-      <c r="F63" s="52" t="n"/>
+      <c r="A63" s="71" t="n"/>
+      <c r="B63" s="72" t="n"/>
+      <c r="C63" s="73" t="n"/>
+      <c r="D63" s="73" t="n"/>
+      <c r="E63" s="73" t="n"/>
+      <c r="F63" s="74" t="n"/>
       <c r="G63" s="52" t="n"/>
-      <c r="H63" s="51" t="n"/>
+      <c r="H63" s="52" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="49" t="n"/>
-      <c r="B64" s="50" t="n"/>
-      <c r="C64" s="52" t="n"/>
-      <c r="D64" s="52" t="n"/>
-      <c r="E64" s="52" t="n"/>
-      <c r="F64" s="52" t="n"/>
+      <c r="A64" s="71" t="n"/>
+      <c r="B64" s="72" t="n"/>
+      <c r="C64" s="73" t="n"/>
+      <c r="D64" s="73" t="n"/>
+      <c r="E64" s="73" t="n"/>
+      <c r="F64" s="74" t="n"/>
       <c r="G64" s="52" t="n"/>
-      <c r="H64" s="51" t="n"/>
+      <c r="H64" s="52" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="49" t="n"/>
-      <c r="B65" s="50" t="n"/>
-      <c r="C65" s="52" t="n"/>
-      <c r="D65" s="52" t="n"/>
-      <c r="E65" s="52" t="n"/>
-      <c r="F65" s="52" t="n"/>
+      <c r="A65" s="71" t="n"/>
+      <c r="B65" s="72" t="n"/>
+      <c r="C65" s="73" t="n"/>
+      <c r="D65" s="73" t="n"/>
+      <c r="E65" s="73" t="n"/>
+      <c r="F65" s="74" t="n"/>
       <c r="G65" s="52" t="n"/>
-      <c r="H65" s="51" t="n"/>
+      <c r="H65" s="52" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="49" t="n"/>
-      <c r="B66" s="50" t="n"/>
-      <c r="C66" s="52" t="n"/>
-      <c r="D66" s="52" t="n"/>
-      <c r="E66" s="52" t="n"/>
-      <c r="F66" s="52" t="n"/>
+      <c r="A66" s="71" t="n"/>
+      <c r="B66" s="72" t="n"/>
+      <c r="C66" s="73" t="n"/>
+      <c r="D66" s="73" t="n"/>
+      <c r="E66" s="73" t="n"/>
+      <c r="F66" s="74" t="n"/>
       <c r="G66" s="52" t="n"/>
-      <c r="H66" s="51" t="n"/>
+      <c r="H66" s="52" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="49" t="n"/>
-      <c r="B67" s="50" t="n"/>
-      <c r="C67" s="52" t="n"/>
-      <c r="D67" s="52" t="n"/>
-      <c r="E67" s="52" t="n"/>
-      <c r="F67" s="52" t="n"/>
+      <c r="A67" s="71" t="n"/>
+      <c r="B67" s="72" t="n"/>
+      <c r="C67" s="73" t="n"/>
+      <c r="D67" s="73" t="n"/>
+      <c r="E67" s="73" t="n"/>
+      <c r="F67" s="74" t="n"/>
       <c r="G67" s="52" t="n"/>
-      <c r="H67" s="51" t="n"/>
+      <c r="H67" s="52" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="49" t="n"/>
-      <c r="B68" s="50" t="n"/>
-      <c r="C68" s="52" t="n"/>
-      <c r="D68" s="52" t="n"/>
-      <c r="E68" s="52" t="n"/>
-      <c r="F68" s="52" t="n"/>
+      <c r="A68" s="71" t="n"/>
+      <c r="B68" s="72" t="n"/>
+      <c r="C68" s="73" t="n"/>
+      <c r="D68" s="73" t="n"/>
+      <c r="E68" s="73" t="n"/>
+      <c r="F68" s="74" t="n"/>
       <c r="G68" s="52" t="n"/>
-      <c r="H68" s="51" t="n"/>
+      <c r="H68" s="52" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="49" t="n"/>
-      <c r="B69" s="50" t="n"/>
-      <c r="C69" s="52" t="n"/>
-      <c r="D69" s="52" t="n"/>
-      <c r="E69" s="52" t="n"/>
-      <c r="F69" s="52" t="n"/>
+      <c r="A69" s="71" t="n"/>
+      <c r="B69" s="72" t="n"/>
+      <c r="C69" s="73" t="n"/>
+      <c r="D69" s="73" t="n"/>
+      <c r="E69" s="73" t="n"/>
+      <c r="F69" s="74" t="n"/>
       <c r="G69" s="52" t="n"/>
-      <c r="H69" s="51" t="n"/>
+      <c r="H69" s="52" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="49" t="n"/>
-      <c r="B70" s="50" t="n"/>
-      <c r="C70" s="52" t="n"/>
-      <c r="D70" s="52" t="n"/>
-      <c r="E70" s="52" t="n"/>
-      <c r="F70" s="52" t="n"/>
+      <c r="A70" s="71" t="n"/>
+      <c r="B70" s="72" t="n"/>
+      <c r="C70" s="73" t="n"/>
+      <c r="D70" s="73" t="n"/>
+      <c r="E70" s="73" t="n"/>
+      <c r="F70" s="74" t="n"/>
       <c r="G70" s="52" t="n"/>
-      <c r="H70" s="51" t="n"/>
+      <c r="H70" s="52" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="49" t="n"/>
-      <c r="B71" s="50" t="n"/>
-      <c r="C71" s="52" t="n"/>
-      <c r="D71" s="52" t="n"/>
-      <c r="E71" s="52" t="n"/>
-      <c r="F71" s="52" t="n"/>
+      <c r="A71" s="71" t="n"/>
+      <c r="B71" s="72" t="n"/>
+      <c r="C71" s="73" t="n"/>
+      <c r="D71" s="73" t="n"/>
+      <c r="E71" s="73" t="n"/>
+      <c r="F71" s="74" t="n"/>
       <c r="G71" s="52" t="n"/>
-      <c r="H71" s="51" t="n"/>
+      <c r="H71" s="52" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="49" t="n"/>
-      <c r="B72" s="50" t="n"/>
-      <c r="C72" s="52" t="n"/>
-      <c r="D72" s="52" t="n"/>
-      <c r="E72" s="52" t="n"/>
-      <c r="F72" s="52" t="n"/>
+      <c r="A72" s="71" t="n"/>
+      <c r="B72" s="72" t="n"/>
+      <c r="C72" s="73" t="n"/>
+      <c r="D72" s="73" t="n"/>
+      <c r="E72" s="73" t="n"/>
+      <c r="F72" s="74" t="n"/>
       <c r="G72" s="52" t="n"/>
-      <c r="H72" s="51" t="n"/>
+      <c r="H72" s="52" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="49" t="n"/>
-      <c r="B73" s="50" t="n"/>
-      <c r="C73" s="52" t="n"/>
-      <c r="D73" s="52" t="n"/>
-      <c r="E73" s="52" t="n"/>
-      <c r="F73" s="52" t="n"/>
+      <c r="A73" s="71" t="n"/>
+      <c r="B73" s="72" t="n"/>
+      <c r="C73" s="73" t="n"/>
+      <c r="D73" s="73" t="n"/>
+      <c r="E73" s="73" t="n"/>
+      <c r="F73" s="74" t="n"/>
       <c r="G73" s="52" t="n"/>
-      <c r="H73" s="51" t="n"/>
+      <c r="H73" s="52" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="49" t="n"/>
-      <c r="B74" s="50" t="n"/>
-      <c r="C74" s="52" t="n"/>
-      <c r="D74" s="52" t="n"/>
-      <c r="E74" s="52" t="n"/>
-      <c r="F74" s="52" t="n"/>
+      <c r="A74" s="71" t="n"/>
+      <c r="B74" s="72" t="n"/>
+      <c r="C74" s="73" t="n"/>
+      <c r="D74" s="73" t="n"/>
+      <c r="E74" s="73" t="n"/>
+      <c r="F74" s="74" t="n"/>
       <c r="G74" s="52" t="n"/>
-      <c r="H74" s="51" t="n"/>
+      <c r="H74" s="52" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="49" t="n"/>
-      <c r="B75" s="50" t="n"/>
-      <c r="C75" s="52" t="n"/>
-      <c r="D75" s="52" t="n"/>
-      <c r="E75" s="52" t="n"/>
-      <c r="F75" s="52" t="n"/>
+      <c r="A75" s="71" t="n"/>
+      <c r="B75" s="72" t="n"/>
+      <c r="C75" s="73" t="n"/>
+      <c r="D75" s="73" t="n"/>
+      <c r="E75" s="73" t="n"/>
+      <c r="F75" s="74" t="n"/>
       <c r="G75" s="52" t="n"/>
-      <c r="H75" s="51" t="n"/>
+      <c r="H75" s="52" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="49" t="n"/>
-      <c r="B76" s="50" t="n"/>
-      <c r="C76" s="52" t="n"/>
-      <c r="D76" s="52" t="n"/>
-      <c r="E76" s="52" t="n"/>
-      <c r="F76" s="52" t="n"/>
+      <c r="A76" s="71" t="n"/>
+      <c r="B76" s="72" t="n"/>
+      <c r="C76" s="73" t="n"/>
+      <c r="D76" s="73" t="n"/>
+      <c r="E76" s="73" t="n"/>
+      <c r="F76" s="74" t="n"/>
       <c r="G76" s="52" t="n"/>
-      <c r="H76" s="51" t="n"/>
+      <c r="H76" s="52" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="49" t="n"/>
-      <c r="B77" s="50" t="n"/>
-      <c r="C77" s="52" t="n"/>
-      <c r="D77" s="52" t="n"/>
-      <c r="E77" s="52" t="n"/>
-      <c r="F77" s="52" t="n"/>
+      <c r="A77" s="71" t="n"/>
+      <c r="B77" s="72" t="n"/>
+      <c r="C77" s="73" t="n"/>
+      <c r="D77" s="73" t="n"/>
+      <c r="E77" s="73" t="n"/>
+      <c r="F77" s="74" t="n"/>
       <c r="G77" s="52" t="n"/>
-      <c r="H77" s="51" t="n"/>
+      <c r="H77" s="52" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="49" t="n"/>
-      <c r="B78" s="50" t="n"/>
-      <c r="C78" s="52" t="n"/>
-      <c r="D78" s="52" t="n"/>
-      <c r="E78" s="52" t="n"/>
-      <c r="F78" s="52" t="n"/>
+      <c r="A78" s="71" t="n"/>
+      <c r="B78" s="72" t="n"/>
+      <c r="C78" s="73" t="n"/>
+      <c r="D78" s="73" t="n"/>
+      <c r="E78" s="73" t="n"/>
+      <c r="F78" s="74" t="n"/>
       <c r="G78" s="52" t="n"/>
-      <c r="H78" s="51" t="n"/>
+      <c r="H78" s="52" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="49" t="n"/>
-      <c r="B79" s="50" t="n"/>
-      <c r="C79" s="52" t="n"/>
-      <c r="D79" s="52" t="n"/>
-      <c r="E79" s="52" t="n"/>
-      <c r="F79" s="52" t="n"/>
+      <c r="A79" s="71" t="n"/>
+      <c r="B79" s="72" t="n"/>
+      <c r="C79" s="73" t="n"/>
+      <c r="D79" s="73" t="n"/>
+      <c r="E79" s="73" t="n"/>
+      <c r="F79" s="74" t="n"/>
       <c r="G79" s="52" t="n"/>
-      <c r="H79" s="51" t="n"/>
+      <c r="H79" s="52" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="49" t="n"/>
-      <c r="B80" s="50" t="n"/>
-      <c r="C80" s="52" t="n"/>
-      <c r="D80" s="52" t="n"/>
-      <c r="E80" s="52" t="n"/>
-      <c r="F80" s="52" t="n"/>
+      <c r="A80" s="71" t="n"/>
+      <c r="B80" s="72" t="n"/>
+      <c r="C80" s="73" t="n"/>
+      <c r="D80" s="73" t="n"/>
+      <c r="E80" s="73" t="n"/>
+      <c r="F80" s="74" t="n"/>
       <c r="G80" s="52" t="n"/>
-      <c r="H80" s="51" t="n"/>
+      <c r="H80" s="52" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="49" t="n"/>
-      <c r="B81" s="50" t="n"/>
-      <c r="C81" s="52" t="n"/>
-      <c r="D81" s="52" t="n"/>
-      <c r="E81" s="52" t="n"/>
-      <c r="F81" s="52" t="n"/>
+      <c r="A81" s="71" t="n"/>
+      <c r="B81" s="72" t="n"/>
+      <c r="C81" s="73" t="n"/>
+      <c r="D81" s="73" t="n"/>
+      <c r="E81" s="73" t="n"/>
+      <c r="F81" s="74" t="n"/>
       <c r="G81" s="52" t="n"/>
-      <c r="H81" s="51" t="n"/>
+      <c r="H81" s="52" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="49" t="n"/>
-      <c r="B82" s="50" t="n"/>
-      <c r="C82" s="52" t="n"/>
-      <c r="D82" s="52" t="n"/>
-      <c r="E82" s="52" t="n"/>
-      <c r="F82" s="52" t="n"/>
+      <c r="A82" s="71" t="n"/>
+      <c r="B82" s="72" t="n"/>
+      <c r="C82" s="73" t="n"/>
+      <c r="D82" s="73" t="n"/>
+      <c r="E82" s="73" t="n"/>
+      <c r="F82" s="74" t="n"/>
       <c r="G82" s="52" t="n"/>
-      <c r="H82" s="51" t="n"/>
+      <c r="H82" s="52" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="49" t="n"/>
-      <c r="B83" s="50" t="n"/>
-      <c r="C83" s="52" t="n"/>
-      <c r="D83" s="52" t="n"/>
-      <c r="E83" s="52" t="n"/>
-      <c r="F83" s="52" t="n"/>
+      <c r="A83" s="71" t="n"/>
+      <c r="B83" s="72" t="n"/>
+      <c r="C83" s="73" t="n"/>
+      <c r="D83" s="73" t="n"/>
+      <c r="E83" s="73" t="n"/>
+      <c r="F83" s="74" t="n"/>
       <c r="G83" s="52" t="n"/>
-      <c r="H83" s="51" t="n"/>
+      <c r="H83" s="52" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="49" t="n"/>
-      <c r="B84" s="50" t="n"/>
-      <c r="C84" s="52" t="n"/>
-      <c r="D84" s="52" t="n"/>
-      <c r="E84" s="52" t="n"/>
-      <c r="F84" s="52" t="n"/>
+      <c r="A84" s="71" t="n"/>
+      <c r="B84" s="72" t="n"/>
+      <c r="C84" s="73" t="n"/>
+      <c r="D84" s="73" t="n"/>
+      <c r="E84" s="73" t="n"/>
+      <c r="F84" s="74" t="n"/>
       <c r="G84" s="52" t="n"/>
-      <c r="H84" s="51" t="n"/>
+      <c r="H84" s="52" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="49" t="n"/>
-      <c r="B85" s="50" t="n"/>
-      <c r="C85" s="52" t="n"/>
-      <c r="D85" s="52" t="n"/>
-      <c r="E85" s="52" t="n"/>
-      <c r="F85" s="52" t="n"/>
+      <c r="A85" s="71" t="n"/>
+      <c r="B85" s="72" t="n"/>
+      <c r="C85" s="73" t="n"/>
+      <c r="D85" s="73" t="n"/>
+      <c r="E85" s="73" t="n"/>
+      <c r="F85" s="74" t="n"/>
       <c r="G85" s="52" t="n"/>
-      <c r="H85" s="51" t="n"/>
+      <c r="H85" s="52" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="49" t="n"/>
-      <c r="B86" s="50" t="n"/>
-      <c r="C86" s="52" t="n"/>
-      <c r="D86" s="52" t="n"/>
-      <c r="E86" s="52" t="n"/>
-      <c r="F86" s="52" t="n"/>
+      <c r="A86" s="71" t="n"/>
+      <c r="B86" s="72" t="n"/>
+      <c r="C86" s="73" t="n"/>
+      <c r="D86" s="73" t="n"/>
+      <c r="E86" s="73" t="n"/>
+      <c r="F86" s="74" t="n"/>
       <c r="G86" s="52" t="n"/>
-      <c r="H86" s="51" t="n"/>
+      <c r="H86" s="52" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="49" t="n"/>
-      <c r="B87" s="50" t="n"/>
-      <c r="C87" s="52" t="n"/>
-      <c r="D87" s="52" t="n"/>
-      <c r="E87" s="52" t="n"/>
-      <c r="F87" s="52" t="n"/>
+      <c r="A87" s="71" t="n"/>
+      <c r="B87" s="72" t="n"/>
+      <c r="C87" s="73" t="n"/>
+      <c r="D87" s="73" t="n"/>
+      <c r="E87" s="73" t="n"/>
+      <c r="F87" s="74" t="n"/>
       <c r="G87" s="52" t="n"/>
-      <c r="H87" s="51" t="n"/>
+      <c r="H87" s="52" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="49" t="n"/>
-      <c r="B88" s="50" t="n"/>
-      <c r="C88" s="52" t="n"/>
-      <c r="D88" s="52" t="n"/>
-      <c r="E88" s="52" t="n"/>
-      <c r="F88" s="52" t="n"/>
+      <c r="A88" s="71" t="n"/>
+      <c r="B88" s="72" t="n"/>
+      <c r="C88" s="73" t="n"/>
+      <c r="D88" s="73" t="n"/>
+      <c r="E88" s="73" t="n"/>
+      <c r="F88" s="74" t="n"/>
       <c r="G88" s="52" t="n"/>
-      <c r="H88" s="51" t="n"/>
+      <c r="H88" s="52" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="49" t="n"/>
-      <c r="B89" s="50" t="n"/>
-      <c r="C89" s="52" t="n"/>
-      <c r="D89" s="52" t="n"/>
-      <c r="E89" s="52" t="n"/>
-      <c r="F89" s="52" t="n"/>
+      <c r="A89" s="71" t="n"/>
+      <c r="B89" s="72" t="n"/>
+      <c r="C89" s="73" t="n"/>
+      <c r="D89" s="73" t="n"/>
+      <c r="E89" s="73" t="n"/>
+      <c r="F89" s="74" t="n"/>
       <c r="G89" s="52" t="n"/>
-      <c r="H89" s="51" t="n"/>
+      <c r="H89" s="52" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="49" t="n"/>
-      <c r="B90" s="50" t="n"/>
-      <c r="C90" s="52" t="n"/>
-      <c r="D90" s="52" t="n"/>
-      <c r="E90" s="52" t="n"/>
-      <c r="F90" s="52" t="n"/>
+      <c r="A90" s="71" t="n"/>
+      <c r="B90" s="72" t="n"/>
+      <c r="C90" s="73" t="n"/>
+      <c r="D90" s="73" t="n"/>
+      <c r="E90" s="73" t="n"/>
+      <c r="F90" s="74" t="n"/>
       <c r="G90" s="52" t="n"/>
-      <c r="H90" s="51" t="n"/>
+      <c r="H90" s="52" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="49" t="n"/>
-      <c r="B91" s="50" t="n"/>
-      <c r="C91" s="52" t="n"/>
-      <c r="D91" s="52" t="n"/>
-      <c r="E91" s="52" t="n"/>
-      <c r="F91" s="52" t="n"/>
+      <c r="A91" s="71" t="n"/>
+      <c r="B91" s="72" t="n"/>
+      <c r="C91" s="73" t="n"/>
+      <c r="D91" s="73" t="n"/>
+      <c r="E91" s="73" t="n"/>
+      <c r="F91" s="74" t="n"/>
       <c r="G91" s="52" t="n"/>
-      <c r="H91" s="51" t="n"/>
+      <c r="H91" s="52" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="49" t="n"/>
-      <c r="B92" s="50" t="n"/>
-      <c r="C92" s="52" t="n"/>
-      <c r="D92" s="52" t="n"/>
-      <c r="E92" s="52" t="n"/>
-      <c r="F92" s="52" t="n"/>
+      <c r="A92" s="71" t="n"/>
+      <c r="B92" s="72" t="n"/>
+      <c r="C92" s="73" t="n"/>
+      <c r="D92" s="73" t="n"/>
+      <c r="E92" s="73" t="n"/>
+      <c r="F92" s="74" t="n"/>
       <c r="G92" s="52" t="n"/>
-      <c r="H92" s="51" t="n"/>
+      <c r="H92" s="52" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="49" t="n"/>
-      <c r="B93" s="50" t="n"/>
-      <c r="C93" s="52" t="n"/>
-      <c r="D93" s="52" t="n"/>
-      <c r="E93" s="52" t="n"/>
-      <c r="F93" s="52" t="n"/>
+      <c r="A93" s="71" t="n"/>
+      <c r="B93" s="72" t="n"/>
+      <c r="C93" s="73" t="n"/>
+      <c r="D93" s="73" t="n"/>
+      <c r="E93" s="73" t="n"/>
+      <c r="F93" s="74" t="n"/>
       <c r="G93" s="52" t="n"/>
-      <c r="H93" s="51" t="n"/>
+      <c r="H93" s="52" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="49" t="n"/>
-      <c r="B94" s="50" t="n"/>
-      <c r="C94" s="52" t="n"/>
-      <c r="D94" s="52" t="n"/>
-      <c r="E94" s="52" t="n"/>
-      <c r="F94" s="52" t="n"/>
+      <c r="A94" s="71" t="n"/>
+      <c r="B94" s="72" t="n"/>
+      <c r="C94" s="73" t="n"/>
+      <c r="D94" s="73" t="n"/>
+      <c r="E94" s="73" t="n"/>
+      <c r="F94" s="74" t="n"/>
       <c r="G94" s="52" t="n"/>
-      <c r="H94" s="51" t="n"/>
+      <c r="H94" s="52" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="49" t="n"/>
-      <c r="B95" s="50" t="n"/>
-      <c r="C95" s="52" t="n"/>
-      <c r="D95" s="52" t="n"/>
-      <c r="E95" s="52" t="n"/>
-      <c r="F95" s="52" t="n"/>
+      <c r="A95" s="71" t="n"/>
+      <c r="B95" s="72" t="n"/>
+      <c r="C95" s="73" t="n"/>
+      <c r="D95" s="73" t="n"/>
+      <c r="E95" s="73" t="n"/>
+      <c r="F95" s="74" t="n"/>
       <c r="G95" s="52" t="n"/>
-      <c r="H95" s="51" t="n"/>
+      <c r="H95" s="52" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="49" t="n"/>
-      <c r="B96" s="50" t="n"/>
-      <c r="C96" s="52" t="n"/>
-      <c r="D96" s="52" t="n"/>
-      <c r="E96" s="52" t="n"/>
-      <c r="F96" s="52" t="n"/>
+      <c r="A96" s="71" t="n"/>
+      <c r="B96" s="72" t="n"/>
+      <c r="C96" s="73" t="n"/>
+      <c r="D96" s="73" t="n"/>
+      <c r="E96" s="73" t="n"/>
+      <c r="F96" s="74" t="n"/>
       <c r="G96" s="52" t="n"/>
-      <c r="H96" s="51" t="n"/>
+      <c r="H96" s="52" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="49" t="n"/>
-      <c r="B97" s="50" t="n"/>
-      <c r="C97" s="52" t="n"/>
-      <c r="D97" s="52" t="n"/>
-      <c r="E97" s="52" t="n"/>
-      <c r="F97" s="52" t="n"/>
+      <c r="A97" s="71" t="n"/>
+      <c r="B97" s="72" t="n"/>
+      <c r="C97" s="73" t="n"/>
+      <c r="D97" s="73" t="n"/>
+      <c r="E97" s="73" t="n"/>
+      <c r="F97" s="74" t="n"/>
       <c r="G97" s="52" t="n"/>
-      <c r="H97" s="51" t="n"/>
+      <c r="H97" s="52" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="49" t="n"/>
-      <c r="B98" s="50" t="n"/>
-      <c r="C98" s="52" t="n"/>
-      <c r="D98" s="52" t="n"/>
-      <c r="E98" s="52" t="n"/>
-      <c r="F98" s="52" t="n"/>
+      <c r="A98" s="71" t="n"/>
+      <c r="B98" s="72" t="n"/>
+      <c r="C98" s="73" t="n"/>
+      <c r="D98" s="73" t="n"/>
+      <c r="E98" s="73" t="n"/>
+      <c r="F98" s="74" t="n"/>
       <c r="G98" s="52" t="n"/>
-      <c r="H98" s="51" t="n"/>
+      <c r="H98" s="52" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="49" t="n"/>
-      <c r="B99" s="50" t="n"/>
-      <c r="C99" s="52" t="n"/>
-      <c r="D99" s="52" t="n"/>
-      <c r="E99" s="52" t="n"/>
-      <c r="F99" s="52" t="n"/>
+      <c r="A99" s="71" t="n"/>
+      <c r="B99" s="72" t="n"/>
+      <c r="C99" s="73" t="n"/>
+      <c r="D99" s="73" t="n"/>
+      <c r="E99" s="73" t="n"/>
+      <c r="F99" s="74" t="n"/>
       <c r="G99" s="52" t="n"/>
-      <c r="H99" s="51" t="n"/>
+      <c r="H99" s="52" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="49" t="n"/>
-      <c r="B100" s="50" t="n"/>
-      <c r="C100" s="52" t="n"/>
-      <c r="D100" s="52" t="n"/>
-      <c r="E100" s="52" t="n"/>
-      <c r="F100" s="52" t="n"/>
+      <c r="A100" s="71" t="n"/>
+      <c r="B100" s="72" t="n"/>
+      <c r="C100" s="73" t="n"/>
+      <c r="D100" s="73" t="n"/>
+      <c r="E100" s="73" t="n"/>
+      <c r="F100" s="74" t="n"/>
       <c r="G100" s="52" t="n"/>
-      <c r="H100" s="51" t="n"/>
+      <c r="H100" s="52" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="49" t="n"/>
-      <c r="B101" s="50" t="n"/>
-      <c r="C101" s="52" t="n"/>
-      <c r="D101" s="52" t="n"/>
-      <c r="E101" s="52" t="n"/>
-      <c r="F101" s="52" t="n"/>
+      <c r="A101" s="71" t="n"/>
+      <c r="B101" s="72" t="n"/>
+      <c r="C101" s="73" t="n"/>
+      <c r="D101" s="73" t="n"/>
+      <c r="E101" s="73" t="n"/>
+      <c r="F101" s="74" t="n"/>
       <c r="G101" s="52" t="n"/>
-      <c r="H101" s="51" t="n"/>
+      <c r="H101" s="52" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="49" t="n"/>
-      <c r="B102" s="50" t="n"/>
-      <c r="C102" s="52" t="n"/>
-      <c r="D102" s="52" t="n"/>
-      <c r="E102" s="52" t="n"/>
-      <c r="F102" s="52" t="n"/>
+      <c r="A102" s="71" t="n"/>
+      <c r="B102" s="72" t="n"/>
+      <c r="C102" s="73" t="n"/>
+      <c r="D102" s="73" t="n"/>
+      <c r="E102" s="73" t="n"/>
+      <c r="F102" s="74" t="n"/>
       <c r="G102" s="52" t="n"/>
-      <c r="H102" s="51" t="n"/>
+      <c r="H102" s="52" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="BB24"/>
   <dataValidations count="6">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Kosongkan untuk siswa baru. Pertahankan ID untuk mengedit siswa." promptTitle="ID siswa" prompt="Kosongkan untuk siswa baru. Pertahankan ID untuk mengedit siswa." type="custom" errorStyle="stop" operator="between">
       <formula1>OR(A2="",AND(ISNUMBER(A2),A2=INT(A2),A2&gt;=1,COUNTIF($A$2:$A$1048576,A2)=1))</formula1>
@@ -2461,7 +2521,7 @@
       <formula1>1</formula1>
       <formula2>255</formula2>
     </dataValidation>
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." promptTitle="ID kelas" prompt="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." promptTitle="ID kelas" prompt="Isi ID kelas yang sudah ada, atau kosongkan jika belum memiliki kelas." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2521,510 +2581,511 @@
     </row>
     <row r="2" ht="24" customFormat="1" customHeight="1" s="21">
       <c r="A2" s="59" t="n"/>
-      <c r="B2" s="60" t="n"/>
-      <c r="C2" s="61" t="n"/>
+      <c r="B2" s="75" t="n"/>
+      <c r="C2" s="76" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="59" t="n"/>
-      <c r="B3" s="60" t="n"/>
-      <c r="C3" s="61" t="n"/>
+      <c r="B3" s="75" t="n"/>
+      <c r="C3" s="76" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="59" t="n"/>
-      <c r="B4" s="60" t="n"/>
-      <c r="C4" s="61" t="n"/>
+      <c r="B4" s="75" t="n"/>
+      <c r="C4" s="76" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="59" t="n"/>
-      <c r="B5" s="60" t="n"/>
-      <c r="C5" s="61" t="n"/>
+      <c r="B5" s="75" t="n"/>
+      <c r="C5" s="76" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="59" t="n"/>
-      <c r="B6" s="60" t="n"/>
-      <c r="C6" s="61" t="n"/>
+      <c r="B6" s="75" t="n"/>
+      <c r="C6" s="76" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="59" t="n"/>
-      <c r="B7" s="60" t="n"/>
-      <c r="C7" s="61" t="n"/>
+      <c r="B7" s="75" t="n"/>
+      <c r="C7" s="76" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="59" t="n"/>
-      <c r="B8" s="60" t="n"/>
-      <c r="C8" s="61" t="n"/>
+      <c r="B8" s="75" t="n"/>
+      <c r="C8" s="76" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="59" t="n"/>
-      <c r="B9" s="60" t="n"/>
-      <c r="C9" s="61" t="n"/>
+      <c r="B9" s="75" t="n"/>
+      <c r="C9" s="76" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="59" t="n"/>
-      <c r="B10" s="60" t="n"/>
-      <c r="C10" s="61" t="n"/>
+      <c r="B10" s="75" t="n"/>
+      <c r="C10" s="76" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="59" t="n"/>
-      <c r="B11" s="60" t="n"/>
-      <c r="C11" s="61" t="n"/>
+      <c r="B11" s="75" t="n"/>
+      <c r="C11" s="76" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="59" t="n"/>
-      <c r="B12" s="60" t="n"/>
-      <c r="C12" s="61" t="n"/>
+      <c r="B12" s="75" t="n"/>
+      <c r="C12" s="76" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="59" t="n"/>
-      <c r="B13" s="60" t="n"/>
-      <c r="C13" s="61" t="n"/>
+      <c r="B13" s="75" t="n"/>
+      <c r="C13" s="76" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="59" t="n"/>
-      <c r="B14" s="60" t="n"/>
-      <c r="C14" s="61" t="n"/>
+      <c r="B14" s="75" t="n"/>
+      <c r="C14" s="76" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="59" t="n"/>
-      <c r="B15" s="60" t="n"/>
-      <c r="C15" s="61" t="n"/>
+      <c r="B15" s="75" t="n"/>
+      <c r="C15" s="76" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="59" t="n"/>
-      <c r="B16" s="60" t="n"/>
-      <c r="C16" s="61" t="n"/>
+      <c r="B16" s="75" t="n"/>
+      <c r="C16" s="76" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="59" t="n"/>
-      <c r="B17" s="60" t="n"/>
-      <c r="C17" s="61" t="n"/>
+      <c r="B17" s="75" t="n"/>
+      <c r="C17" s="76" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="59" t="n"/>
-      <c r="B18" s="60" t="n"/>
-      <c r="C18" s="61" t="n"/>
+      <c r="B18" s="75" t="n"/>
+      <c r="C18" s="76" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="59" t="n"/>
-      <c r="B19" s="60" t="n"/>
-      <c r="C19" s="61" t="n"/>
+      <c r="B19" s="75" t="n"/>
+      <c r="C19" s="76" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="59" t="n"/>
-      <c r="B20" s="60" t="n"/>
-      <c r="C20" s="61" t="n"/>
+      <c r="B20" s="75" t="n"/>
+      <c r="C20" s="76" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="59" t="n"/>
-      <c r="B21" s="60" t="n"/>
-      <c r="C21" s="61" t="n"/>
+      <c r="B21" s="75" t="n"/>
+      <c r="C21" s="76" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="59" t="n"/>
-      <c r="B22" s="60" t="n"/>
-      <c r="C22" s="61" t="n"/>
+      <c r="B22" s="75" t="n"/>
+      <c r="C22" s="76" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="59" t="n"/>
-      <c r="B23" s="60" t="n"/>
-      <c r="C23" s="61" t="n"/>
+      <c r="B23" s="75" t="n"/>
+      <c r="C23" s="76" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="59" t="n"/>
-      <c r="B24" s="60" t="n"/>
-      <c r="C24" s="61" t="n"/>
+      <c r="B24" s="75" t="n"/>
+      <c r="C24" s="76" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="59" t="n"/>
-      <c r="B25" s="60" t="n"/>
-      <c r="C25" s="61" t="n"/>
+      <c r="B25" s="75" t="n"/>
+      <c r="C25" s="76" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="59" t="n"/>
-      <c r="B26" s="60" t="n"/>
-      <c r="C26" s="61" t="n"/>
+      <c r="B26" s="75" t="n"/>
+      <c r="C26" s="76" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="59" t="n"/>
-      <c r="B27" s="60" t="n"/>
-      <c r="C27" s="61" t="n"/>
+      <c r="B27" s="75" t="n"/>
+      <c r="C27" s="76" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="59" t="n"/>
-      <c r="B28" s="60" t="n"/>
-      <c r="C28" s="61" t="n"/>
+      <c r="B28" s="75" t="n"/>
+      <c r="C28" s="76" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="59" t="n"/>
-      <c r="B29" s="60" t="n"/>
-      <c r="C29" s="61" t="n"/>
+      <c r="B29" s="75" t="n"/>
+      <c r="C29" s="76" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="59" t="n"/>
-      <c r="B30" s="60" t="n"/>
-      <c r="C30" s="61" t="n"/>
+      <c r="B30" s="75" t="n"/>
+      <c r="C30" s="76" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="59" t="n"/>
-      <c r="B31" s="60" t="n"/>
-      <c r="C31" s="61" t="n"/>
+      <c r="B31" s="75" t="n"/>
+      <c r="C31" s="76" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="59" t="n"/>
-      <c r="B32" s="60" t="n"/>
-      <c r="C32" s="61" t="n"/>
+      <c r="B32" s="75" t="n"/>
+      <c r="C32" s="76" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="59" t="n"/>
-      <c r="B33" s="60" t="n"/>
-      <c r="C33" s="61" t="n"/>
+      <c r="B33" s="75" t="n"/>
+      <c r="C33" s="76" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="59" t="n"/>
-      <c r="B34" s="60" t="n"/>
-      <c r="C34" s="61" t="n"/>
+      <c r="B34" s="75" t="n"/>
+      <c r="C34" s="76" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="59" t="n"/>
-      <c r="B35" s="60" t="n"/>
-      <c r="C35" s="61" t="n"/>
+      <c r="B35" s="75" t="n"/>
+      <c r="C35" s="76" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="59" t="n"/>
-      <c r="B36" s="60" t="n"/>
-      <c r="C36" s="61" t="n"/>
+      <c r="B36" s="75" t="n"/>
+      <c r="C36" s="76" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="59" t="n"/>
-      <c r="B37" s="60" t="n"/>
-      <c r="C37" s="61" t="n"/>
+      <c r="B37" s="75" t="n"/>
+      <c r="C37" s="76" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="59" t="n"/>
-      <c r="B38" s="60" t="n"/>
-      <c r="C38" s="61" t="n"/>
+      <c r="B38" s="75" t="n"/>
+      <c r="C38" s="76" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="59" t="n"/>
-      <c r="B39" s="60" t="n"/>
-      <c r="C39" s="61" t="n"/>
+      <c r="B39" s="75" t="n"/>
+      <c r="C39" s="76" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="59" t="n"/>
-      <c r="B40" s="60" t="n"/>
-      <c r="C40" s="61" t="n"/>
+      <c r="B40" s="75" t="n"/>
+      <c r="C40" s="76" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="59" t="n"/>
-      <c r="B41" s="60" t="n"/>
-      <c r="C41" s="61" t="n"/>
+      <c r="B41" s="75" t="n"/>
+      <c r="C41" s="76" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="59" t="n"/>
-      <c r="B42" s="60" t="n"/>
-      <c r="C42" s="61" t="n"/>
+      <c r="B42" s="75" t="n"/>
+      <c r="C42" s="76" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="59" t="n"/>
-      <c r="B43" s="60" t="n"/>
-      <c r="C43" s="61" t="n"/>
+      <c r="B43" s="75" t="n"/>
+      <c r="C43" s="76" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="59" t="n"/>
-      <c r="B44" s="60" t="n"/>
-      <c r="C44" s="61" t="n"/>
+      <c r="B44" s="75" t="n"/>
+      <c r="C44" s="76" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="59" t="n"/>
-      <c r="B45" s="60" t="n"/>
-      <c r="C45" s="61" t="n"/>
+      <c r="B45" s="75" t="n"/>
+      <c r="C45" s="76" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="59" t="n"/>
-      <c r="B46" s="60" t="n"/>
-      <c r="C46" s="61" t="n"/>
+      <c r="B46" s="75" t="n"/>
+      <c r="C46" s="76" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="59" t="n"/>
-      <c r="B47" s="60" t="n"/>
-      <c r="C47" s="61" t="n"/>
+      <c r="B47" s="75" t="n"/>
+      <c r="C47" s="76" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="59" t="n"/>
-      <c r="B48" s="60" t="n"/>
-      <c r="C48" s="61" t="n"/>
+      <c r="B48" s="75" t="n"/>
+      <c r="C48" s="76" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="59" t="n"/>
-      <c r="B49" s="60" t="n"/>
-      <c r="C49" s="61" t="n"/>
+      <c r="B49" s="75" t="n"/>
+      <c r="C49" s="76" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="59" t="n"/>
-      <c r="B50" s="60" t="n"/>
-      <c r="C50" s="61" t="n"/>
+      <c r="B50" s="75" t="n"/>
+      <c r="C50" s="76" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="59" t="n"/>
-      <c r="B51" s="60" t="n"/>
-      <c r="C51" s="61" t="n"/>
+      <c r="B51" s="75" t="n"/>
+      <c r="C51" s="76" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="59" t="n"/>
-      <c r="B52" s="60" t="n"/>
-      <c r="C52" s="61" t="n"/>
+      <c r="B52" s="75" t="n"/>
+      <c r="C52" s="76" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="59" t="n"/>
-      <c r="B53" s="60" t="n"/>
-      <c r="C53" s="61" t="n"/>
+      <c r="B53" s="75" t="n"/>
+      <c r="C53" s="76" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="59" t="n"/>
-      <c r="B54" s="60" t="n"/>
-      <c r="C54" s="61" t="n"/>
+      <c r="B54" s="75" t="n"/>
+      <c r="C54" s="76" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="59" t="n"/>
-      <c r="B55" s="60" t="n"/>
-      <c r="C55" s="61" t="n"/>
+      <c r="B55" s="75" t="n"/>
+      <c r="C55" s="76" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="59" t="n"/>
-      <c r="B56" s="60" t="n"/>
-      <c r="C56" s="61" t="n"/>
+      <c r="B56" s="75" t="n"/>
+      <c r="C56" s="76" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="59" t="n"/>
-      <c r="B57" s="60" t="n"/>
-      <c r="C57" s="61" t="n"/>
+      <c r="B57" s="75" t="n"/>
+      <c r="C57" s="76" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="59" t="n"/>
-      <c r="B58" s="60" t="n"/>
-      <c r="C58" s="61" t="n"/>
+      <c r="B58" s="75" t="n"/>
+      <c r="C58" s="76" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="59" t="n"/>
-      <c r="B59" s="60" t="n"/>
-      <c r="C59" s="61" t="n"/>
+      <c r="B59" s="75" t="n"/>
+      <c r="C59" s="76" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="59" t="n"/>
-      <c r="B60" s="60" t="n"/>
-      <c r="C60" s="61" t="n"/>
+      <c r="B60" s="75" t="n"/>
+      <c r="C60" s="76" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="59" t="n"/>
-      <c r="B61" s="60" t="n"/>
-      <c r="C61" s="61" t="n"/>
+      <c r="B61" s="75" t="n"/>
+      <c r="C61" s="76" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="59" t="n"/>
-      <c r="B62" s="60" t="n"/>
-      <c r="C62" s="61" t="n"/>
+      <c r="B62" s="75" t="n"/>
+      <c r="C62" s="76" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="59" t="n"/>
-      <c r="B63" s="60" t="n"/>
-      <c r="C63" s="61" t="n"/>
+      <c r="B63" s="75" t="n"/>
+      <c r="C63" s="76" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="59" t="n"/>
-      <c r="B64" s="60" t="n"/>
-      <c r="C64" s="61" t="n"/>
+      <c r="B64" s="75" t="n"/>
+      <c r="C64" s="76" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="59" t="n"/>
-      <c r="B65" s="60" t="n"/>
-      <c r="C65" s="61" t="n"/>
+      <c r="B65" s="75" t="n"/>
+      <c r="C65" s="76" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="59" t="n"/>
-      <c r="B66" s="60" t="n"/>
-      <c r="C66" s="61" t="n"/>
+      <c r="B66" s="75" t="n"/>
+      <c r="C66" s="76" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="59" t="n"/>
-      <c r="B67" s="60" t="n"/>
-      <c r="C67" s="61" t="n"/>
+      <c r="B67" s="75" t="n"/>
+      <c r="C67" s="76" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="59" t="n"/>
-      <c r="B68" s="60" t="n"/>
-      <c r="C68" s="61" t="n"/>
+      <c r="B68" s="75" t="n"/>
+      <c r="C68" s="76" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="59" t="n"/>
-      <c r="B69" s="60" t="n"/>
-      <c r="C69" s="61" t="n"/>
+      <c r="B69" s="75" t="n"/>
+      <c r="C69" s="76" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="59" t="n"/>
-      <c r="B70" s="60" t="n"/>
-      <c r="C70" s="61" t="n"/>
+      <c r="B70" s="75" t="n"/>
+      <c r="C70" s="76" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="59" t="n"/>
-      <c r="B71" s="60" t="n"/>
-      <c r="C71" s="61" t="n"/>
+      <c r="B71" s="75" t="n"/>
+      <c r="C71" s="76" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="59" t="n"/>
-      <c r="B72" s="60" t="n"/>
-      <c r="C72" s="61" t="n"/>
+      <c r="B72" s="75" t="n"/>
+      <c r="C72" s="76" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="59" t="n"/>
-      <c r="B73" s="60" t="n"/>
-      <c r="C73" s="61" t="n"/>
+      <c r="B73" s="75" t="n"/>
+      <c r="C73" s="76" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="59" t="n"/>
-      <c r="B74" s="60" t="n"/>
-      <c r="C74" s="61" t="n"/>
+      <c r="B74" s="75" t="n"/>
+      <c r="C74" s="76" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="59" t="n"/>
-      <c r="B75" s="60" t="n"/>
-      <c r="C75" s="61" t="n"/>
+      <c r="B75" s="75" t="n"/>
+      <c r="C75" s="76" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="59" t="n"/>
-      <c r="B76" s="60" t="n"/>
-      <c r="C76" s="61" t="n"/>
+      <c r="B76" s="75" t="n"/>
+      <c r="C76" s="76" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="59" t="n"/>
-      <c r="B77" s="60" t="n"/>
-      <c r="C77" s="61" t="n"/>
+      <c r="B77" s="75" t="n"/>
+      <c r="C77" s="76" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="59" t="n"/>
-      <c r="B78" s="60" t="n"/>
-      <c r="C78" s="61" t="n"/>
+      <c r="B78" s="75" t="n"/>
+      <c r="C78" s="76" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="59" t="n"/>
-      <c r="B79" s="60" t="n"/>
-      <c r="C79" s="61" t="n"/>
+      <c r="B79" s="75" t="n"/>
+      <c r="C79" s="76" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="59" t="n"/>
-      <c r="B80" s="60" t="n"/>
-      <c r="C80" s="61" t="n"/>
+      <c r="B80" s="75" t="n"/>
+      <c r="C80" s="76" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="59" t="n"/>
-      <c r="B81" s="60" t="n"/>
-      <c r="C81" s="61" t="n"/>
+      <c r="B81" s="75" t="n"/>
+      <c r="C81" s="76" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="59" t="n"/>
-      <c r="B82" s="60" t="n"/>
-      <c r="C82" s="61" t="n"/>
+      <c r="B82" s="75" t="n"/>
+      <c r="C82" s="76" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="59" t="n"/>
-      <c r="B83" s="60" t="n"/>
-      <c r="C83" s="61" t="n"/>
+      <c r="B83" s="75" t="n"/>
+      <c r="C83" s="76" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="59" t="n"/>
-      <c r="B84" s="60" t="n"/>
-      <c r="C84" s="61" t="n"/>
+      <c r="B84" s="75" t="n"/>
+      <c r="C84" s="76" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="59" t="n"/>
-      <c r="B85" s="60" t="n"/>
-      <c r="C85" s="61" t="n"/>
+      <c r="B85" s="75" t="n"/>
+      <c r="C85" s="76" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="59" t="n"/>
-      <c r="B86" s="60" t="n"/>
-      <c r="C86" s="61" t="n"/>
+      <c r="B86" s="75" t="n"/>
+      <c r="C86" s="76" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="59" t="n"/>
-      <c r="B87" s="60" t="n"/>
-      <c r="C87" s="61" t="n"/>
+      <c r="B87" s="75" t="n"/>
+      <c r="C87" s="76" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="59" t="n"/>
-      <c r="B88" s="60" t="n"/>
-      <c r="C88" s="61" t="n"/>
+      <c r="B88" s="75" t="n"/>
+      <c r="C88" s="76" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="59" t="n"/>
-      <c r="B89" s="60" t="n"/>
-      <c r="C89" s="61" t="n"/>
+      <c r="B89" s="75" t="n"/>
+      <c r="C89" s="76" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="59" t="n"/>
-      <c r="B90" s="60" t="n"/>
-      <c r="C90" s="61" t="n"/>
+      <c r="B90" s="75" t="n"/>
+      <c r="C90" s="76" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="59" t="n"/>
-      <c r="B91" s="60" t="n"/>
-      <c r="C91" s="61" t="n"/>
+      <c r="B91" s="75" t="n"/>
+      <c r="C91" s="76" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="59" t="n"/>
-      <c r="B92" s="60" t="n"/>
-      <c r="C92" s="61" t="n"/>
+      <c r="B92" s="75" t="n"/>
+      <c r="C92" s="76" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="59" t="n"/>
-      <c r="B93" s="60" t="n"/>
-      <c r="C93" s="61" t="n"/>
+      <c r="B93" s="75" t="n"/>
+      <c r="C93" s="76" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="59" t="n"/>
-      <c r="B94" s="60" t="n"/>
-      <c r="C94" s="61" t="n"/>
+      <c r="B94" s="75" t="n"/>
+      <c r="C94" s="76" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="59" t="n"/>
-      <c r="B95" s="60" t="n"/>
-      <c r="C95" s="61" t="n"/>
+      <c r="B95" s="75" t="n"/>
+      <c r="C95" s="76" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="59" t="n"/>
-      <c r="B96" s="60" t="n"/>
-      <c r="C96" s="61" t="n"/>
+      <c r="B96" s="75" t="n"/>
+      <c r="C96" s="76" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="59" t="n"/>
-      <c r="B97" s="60" t="n"/>
-      <c r="C97" s="61" t="n"/>
+      <c r="B97" s="75" t="n"/>
+      <c r="C97" s="76" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="59" t="n"/>
-      <c r="B98" s="60" t="n"/>
-      <c r="C98" s="61" t="n"/>
+      <c r="B98" s="75" t="n"/>
+      <c r="C98" s="76" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="59" t="n"/>
-      <c r="B99" s="60" t="n"/>
-      <c r="C99" s="61" t="n"/>
+      <c r="B99" s="75" t="n"/>
+      <c r="C99" s="76" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="59" t="n"/>
-      <c r="B100" s="60" t="n"/>
-      <c r="C100" s="61" t="n"/>
+      <c r="B100" s="75" t="n"/>
+      <c r="C100" s="76" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="59" t="n"/>
-      <c r="B101" s="60" t="n"/>
-      <c r="C101" s="61" t="n"/>
+      <c r="B101" s="75" t="n"/>
+      <c r="C101" s="76" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="59" t="n"/>
-      <c r="B102" s="60" t="n"/>
-      <c r="C102" s="61" t="n"/>
+      <c r="B102" s="75" t="n"/>
+      <c r="C102" s="76" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="D2D4"/>
   <dataValidations count="3">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data tidak valid" error="Kosongkan untuk kelas baru. Pertahankan ID untuk mengedit kelas." promptTitle="ID kelas" prompt="Kosongkan untuk kelas baru. Pertahankan ID untuk mengedit kelas." type="custom" errorStyle="stop" operator="between">
       <formula1>OR(A2="",AND(ISNUMBER(A2),A2=INT(A2),A2&gt;=1,COUNTIF($A$2:$A$1048576,A2)=1))</formula1>

</xml_diff>

<commit_message>
docs: documentation link in relevant pages
</commit_message>
<xml_diff>
--- a/web/app/spreadsheet_templates/students_export_template.xlsx
+++ b/web/app/spreadsheet_templates/students_export_template.xlsx
@@ -1036,7 +1036,7 @@
       <c r="A4" s="23" t="n"/>
       <c r="B4" s="66" t="inlineStr">
         <is>
-          <t>Dokumentasi lengkap: https://example.com</t>
+          <t>Panduan impor dan ekspor data (klik untuk membuka)</t>
         </is>
       </c>
       <c r="C4" s="28" t="n"/>
@@ -1430,7 +1430,7 @@
     <mergeCell ref="B28:H28"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" tooltip="Buka panduan impor dan ekspor Absensa" r:id="rId1"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>